<commit_message>
Atualiza vitrine — 13/07/2026 02:06 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>72600</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>1356159.46</v>
@@ -576,7 +576,7 @@
         <v>4261000</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>6818</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>2904840.54</v>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2890.8</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>2458247.78</v>
@@ -639,7 +639,7 @@
         <v>4880000</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>4963</v>
+        <v>49.63</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>2421752.22</v>
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>61.6</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
@@ -705,7 +705,7 @@
         <v>290000</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>4679</v>
+        <v>46.79</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>135673.74</v>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>40.31</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
@@ -771,7 +771,7 @@
         <v>169000</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>4609</v>
+        <v>46.09</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>77881.17999999999</v>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4590</v>
+        <v>40</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
@@ -837,7 +837,7 @@
         <v>186071.2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>4561</v>
+        <v>45.61</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>84853.64999999999</v>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>10165</v>
+        <v>40</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -903,7 +903,7 @@
         <v>186000</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>4493</v>
+        <v>44.93</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>83561.37</v>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>47.15</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -969,7 +969,7 @@
         <v>235000</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>4491</v>
+        <v>44.91</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>105518.88</v>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4031</v>
+        <v>40.31</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
@@ -1035,7 +1035,7 @@
         <v>213000</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>4410</v>
+        <v>44.1</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>93915.42999999999</v>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G10" t="n">
         <v>2</v>
@@ -1101,7 +1101,7 @@
         <v>190000</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>4368</v>
+        <v>43.68</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>82981.35000000001</v>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>42.27</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -1167,7 +1167,7 @@
         <v>182000</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>4342</v>
+        <v>43.42</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>79009.91</v>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4337</v>
+        <v>41.54</v>
       </c>
       <c r="G12" t="n">
         <v>2</v>
@@ -1233,7 +1233,7 @@
         <v>124000</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>4268</v>
+        <v>42.68</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>52919.1</v>
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>40.31</v>
       </c>
       <c r="G13" t="n">
         <v>2</v>
@@ -1299,7 +1299,7 @@
         <v>195000</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>4224</v>
+        <v>42.24</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>82348.78999999999</v>
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>50.17</v>
       </c>
       <c r="G14" t="n">
         <v>2</v>
@@ -1365,7 +1365,7 @@
         <v>217000</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>4224</v>
+        <v>42.24</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>91639.42999999999</v>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>43388</v>
+        <v>433.88</v>
       </c>
       <c r="G15" t="n">
         <v>5</v>
@@ -1431,7 +1431,7 @@
         <v>1420000</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>4200</v>
+        <v>42</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>596301.55</v>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>86.93000000000001</v>
       </c>
       <c r="G16" t="n">
         <v>3</v>
@@ -1497,7 +1497,7 @@
         <v>356000</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>4162</v>
+        <v>41.62</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>148137.19</v>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>4930</v>
+        <v>42.57</v>
       </c>
       <c r="G17" t="n">
         <v>2</v>
@@ -1563,7 +1563,7 @@
         <v>147000</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>4146</v>
+        <v>41.46</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>60936.94</v>
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>5462</v>
+        <v>41.54</v>
       </c>
       <c r="G18" t="n">
         <v>2</v>
@@ -1629,7 +1629,7 @@
         <v>170000</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>69258.92</v>
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>4337</v>
+        <v>41.54</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -1695,7 +1695,7 @@
         <v>180000</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>73332.97</v>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>5462</v>
+        <v>41.54</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -1761,7 +1761,7 @@
         <v>180000</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>73332.97</v>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>4500</v>
+        <v>43.12</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -1827,7 +1827,7 @@
         <v>180000</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>73332.97</v>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>4052</v>
+        <v>37.8</v>
       </c>
       <c r="G22" t="n">
         <v>2</v>
@@ -1893,7 +1893,7 @@
         <v>180000</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>73332.97</v>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>4228</v>
+        <v>41.7</v>
       </c>
       <c r="G23" t="n">
         <v>2</v>
@@ -1959,7 +1959,7 @@
         <v>165000</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>67221.89</v>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>5003</v>
+        <v>43.61</v>
       </c>
       <c r="G24" t="n">
         <v>2</v>
@@ -2025,7 +2025,7 @@
         <v>173000</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>70481.13</v>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G25" t="n">
         <v>2</v>
@@ -2091,7 +2091,7 @@
         <v>180000</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>73332.97</v>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G26" t="n">
         <v>2</v>
@@ -2157,7 +2157,7 @@
         <v>168000</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>68444.11</v>
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>401921</v>
+        <v>40.13</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
@@ -2223,7 +2223,7 @@
         <v>174000</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>70888.53999999999</v>
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>4592</v>
+        <v>40</v>
       </c>
       <c r="G28" t="n">
         <v>2</v>
@@ -2289,7 +2289,7 @@
         <v>170000</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>69258.92</v>
@@ -2343,7 +2343,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>5200</v>
+        <v>40</v>
       </c>
       <c r="G29" t="n">
         <v>2</v>
@@ -2355,7 +2355,7 @@
         <v>175000</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>71295.94</v>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G30" t="n">
         <v>2</v>
@@ -2421,7 +2421,7 @@
         <v>180000</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>73332.97</v>
@@ -2475,7 +2475,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G31" t="n">
         <v>2</v>
@@ -2487,7 +2487,7 @@
         <v>165000</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>67221.89</v>
@@ -2541,7 +2541,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -2553,7 +2553,7 @@
         <v>177000</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>72110.75999999999</v>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G33" t="n">
         <v>2</v>
@@ -2619,7 +2619,7 @@
         <v>180000</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>73332.97</v>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>5200</v>
+        <v>40</v>
       </c>
       <c r="G34" t="n">
         <v>2</v>
@@ -2685,7 +2685,7 @@
         <v>175000</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>71295.94</v>
@@ -2739,7 +2739,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -2751,7 +2751,7 @@
         <v>174260.53</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>70994.67999999999</v>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
@@ -2817,7 +2817,7 @@
         <v>170000</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>69258.92</v>
@@ -2871,7 +2871,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4626</v>
+        <v>40.31</v>
       </c>
       <c r="G37" t="n">
         <v>2</v>
@@ -2883,7 +2883,7 @@
         <v>179000</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>72925.57000000001</v>
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>52.31</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
@@ -2949,7 +2949,7 @@
         <v>172000</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>70073.73</v>
@@ -3003,7 +3003,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>5003</v>
+        <v>43.61</v>
       </c>
       <c r="G39" t="n">
         <v>2</v>
@@ -3015,7 +3015,7 @@
         <v>179500</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>73129.27</v>
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>5200</v>
+        <v>40</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
@@ -3081,7 +3081,7 @@
         <v>175000</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>71295.94</v>
@@ -3135,7 +3135,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -3147,7 +3147,7 @@
         <v>180000</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>73332.97</v>
@@ -3201,7 +3201,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
@@ -3213,7 +3213,7 @@
         <v>177000</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>72110.75999999999</v>
@@ -3267,7 +3267,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>4490</v>
+        <v>40.1</v>
       </c>
       <c r="G43" t="n">
         <v>2</v>
@@ -3279,7 +3279,7 @@
         <v>161700</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>65877.45</v>
@@ -3333,7 +3333,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>4587</v>
+        <v>40</v>
       </c>
       <c r="G44" t="n">
         <v>2</v>
@@ -3345,7 +3345,7 @@
         <v>167000</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>68036.7</v>
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>5008</v>
+        <v>43.61</v>
       </c>
       <c r="G45" t="n">
         <v>2</v>
@@ -3411,7 +3411,7 @@
         <v>178000</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>72518.16</v>
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4738</v>
+        <v>41.51</v>
       </c>
       <c r="G46" t="n">
         <v>2</v>
@@ -3477,7 +3477,7 @@
         <v>183000</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>74555.19</v>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G47" t="n">
         <v>2</v>
@@ -3543,7 +3543,7 @@
         <v>179000</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>72925.57000000001</v>
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>10233</v>
+        <v>40.31</v>
       </c>
       <c r="G48" t="n">
         <v>2</v>
@@ -3609,7 +3609,7 @@
         <v>170000</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>69258.92</v>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G49" t="n">
         <v>2</v>
@@ -3675,7 +3675,7 @@
         <v>170000</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>69258.92</v>
@@ -3729,7 +3729,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G50" t="n">
         <v>2</v>
@@ -3741,7 +3741,7 @@
         <v>170000</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>69258.92</v>
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G51" t="n">
         <v>2</v>
@@ -3807,7 +3807,7 @@
         <v>173686.52</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>70760.83</v>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>5832</v>
+        <v>40</v>
       </c>
       <c r="G52" t="n">
         <v>2</v>
@@ -3873,7 +3873,7 @@
         <v>183000</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>74555.19</v>
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>4587</v>
+        <v>40</v>
       </c>
       <c r="G53" t="n">
         <v>2</v>
@@ -3939,7 +3939,7 @@
         <v>180000</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>73332.97</v>
@@ -3993,7 +3993,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G54" t="n">
         <v>2</v>
@@ -4005,7 +4005,7 @@
         <v>180000</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>73332.97</v>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>4620</v>
+        <v>40.31</v>
       </c>
       <c r="G55" t="n">
         <v>2</v>
@@ -4071,7 +4071,7 @@
         <v>170000</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>69258.92</v>
@@ -4125,7 +4125,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>4759</v>
+        <v>40</v>
       </c>
       <c r="G56" t="n">
         <v>2</v>
@@ -4137,7 +4137,7 @@
         <v>183000</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>74555.19</v>
@@ -4191,7 +4191,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>40.31</v>
       </c>
       <c r="G57" t="n">
         <v>2</v>
@@ -4203,7 +4203,7 @@
         <v>170000</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>69258.92</v>
@@ -4257,7 +4257,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G58" t="n">
         <v>2</v>
@@ -4269,7 +4269,7 @@
         <v>170000</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>69258.92</v>
@@ -4323,7 +4323,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G59" t="n">
         <v>2</v>
@@ -4335,7 +4335,7 @@
         <v>180000</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>73332.97</v>
@@ -4389,7 +4389,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G60" t="n">
         <v>2</v>
@@ -4401,7 +4401,7 @@
         <v>170000</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>69258.92</v>
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G61" t="n">
         <v>2</v>
@@ -4467,7 +4467,7 @@
         <v>170000</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>69258.92</v>
@@ -4521,7 +4521,7 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>4620</v>
+        <v>40.31</v>
       </c>
       <c r="G62" t="n">
         <v>2</v>
@@ -4533,7 +4533,7 @@
         <v>168000</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>68444.11</v>
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>4587</v>
+        <v>40</v>
       </c>
       <c r="G63" t="n">
         <v>2</v>
@@ -4599,7 +4599,7 @@
         <v>168500</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>68647.81</v>
@@ -4653,7 +4653,7 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>4587</v>
+        <v>40</v>
       </c>
       <c r="G64" t="n">
         <v>2</v>
@@ -4665,7 +4665,7 @@
         <v>163500</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>66610.78</v>
@@ -4719,7 +4719,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>4587</v>
+        <v>40</v>
       </c>
       <c r="G65" t="n">
         <v>2</v>
@@ -4731,7 +4731,7 @@
         <v>175000</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>71295.94</v>
@@ -4785,7 +4785,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>63760</v>
+        <v>40</v>
       </c>
       <c r="G66" t="n">
         <v>2</v>
@@ -4797,7 +4797,7 @@
         <v>176000</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>71703.35000000001</v>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G67" t="n">
         <v>2</v>
@@ -4863,7 +4863,7 @@
         <v>172000</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>70073.73</v>
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>4634</v>
+        <v>40.31</v>
       </c>
       <c r="G68" t="n">
         <v>2</v>
@@ -4929,7 +4929,7 @@
         <v>178000</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>72518.16</v>
@@ -4983,7 +4983,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>4988</v>
+        <v>43.51</v>
       </c>
       <c r="G69" t="n">
         <v>2</v>
@@ -4995,7 +4995,7 @@
         <v>165000</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>67221.89</v>
@@ -5049,7 +5049,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>5830</v>
+        <v>49.84</v>
       </c>
       <c r="G70" t="n">
         <v>2</v>
@@ -5061,7 +5061,7 @@
         <v>180000</v>
       </c>
       <c r="J70" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>73332.97</v>
@@ -5115,7 +5115,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0</v>
+        <v>35.1</v>
       </c>
       <c r="G71" t="n">
         <v>1</v>
@@ -5127,7 +5127,7 @@
         <v>175773.78</v>
       </c>
       <c r="J71" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>71611.19</v>
@@ -5181,7 +5181,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>4730</v>
+        <v>47.3</v>
       </c>
       <c r="G72" t="n">
         <v>2</v>
@@ -5193,7 +5193,7 @@
         <v>162000</v>
       </c>
       <c r="J72" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>65999.67</v>
@@ -5247,7 +5247,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>10120</v>
+        <v>38.68</v>
       </c>
       <c r="G73" t="n">
         <v>2</v>
@@ -5259,7 +5259,7 @@
         <v>180000</v>
       </c>
       <c r="J73" s="3" t="n">
-        <v>4075</v>
+        <v>40.75</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>73332.97</v>
@@ -5313,7 +5313,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G74" t="n">
         <v>2</v>
@@ -5325,7 +5325,7 @@
         <v>250000</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>4031</v>
+        <v>40.31</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>100750.78</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>4212</v>
+        <v>40.32</v>
       </c>
       <c r="G75" t="n">
         <v>2</v>
@@ -5391,7 +5391,7 @@
         <v>189000</v>
       </c>
       <c r="J75" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>74765.85000000001</v>
@@ -5445,7 +5445,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>5817</v>
+        <v>41.11</v>
       </c>
       <c r="G76" t="n">
         <v>2</v>
@@ -5457,7 +5457,7 @@
         <v>188000</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>74370.25999999999</v>
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>4567</v>
+        <v>41.11</v>
       </c>
       <c r="G77" t="n">
         <v>2</v>
@@ -5523,7 +5523,7 @@
         <v>205000</v>
       </c>
       <c r="J77" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>81095.23</v>
@@ -5577,7 +5577,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>5016</v>
+        <v>43.61</v>
       </c>
       <c r="G78" t="n">
         <v>2</v>
@@ -5589,7 +5589,7 @@
         <v>188000</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>74370.25999999999</v>
@@ -5643,7 +5643,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>4549</v>
+        <v>38.4</v>
       </c>
       <c r="G79" t="n">
         <v>2</v>
@@ -5655,7 +5655,7 @@
         <v>219756.47</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>86932.69</v>
@@ -5709,7 +5709,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>4457</v>
+        <v>41.7</v>
       </c>
       <c r="G80" t="n">
         <v>2</v>
@@ -5721,7 +5721,7 @@
         <v>220000</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>87029.03</v>
@@ -5775,7 +5775,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G81" t="n">
         <v>2</v>
@@ -5787,7 +5787,7 @@
         <v>185000</v>
       </c>
       <c r="J81" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>73183.5</v>
@@ -5841,7 +5841,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>5004</v>
+        <v>43.61</v>
       </c>
       <c r="G82" t="n">
         <v>2</v>
@@ -5853,7 +5853,7 @@
         <v>205000</v>
       </c>
       <c r="J82" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>81095.23</v>
@@ -5907,7 +5907,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>6282</v>
+        <v>44.83</v>
       </c>
       <c r="G83" t="n">
         <v>2</v>
@@ -5919,7 +5919,7 @@
         <v>190000</v>
       </c>
       <c r="J83" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>75161.42999999999</v>
@@ -5973,7 +5973,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>4626</v>
+        <v>40.31</v>
       </c>
       <c r="G84" t="n">
         <v>2</v>
@@ -5985,7 +5985,7 @@
         <v>184000</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>72787.92</v>
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>5004</v>
+        <v>43.61</v>
       </c>
       <c r="G85" t="n">
         <v>2</v>
@@ -6051,7 +6051,7 @@
         <v>186000</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>73579.09</v>
@@ -6105,7 +6105,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G86" t="n">
         <v>2</v>
@@ -6117,7 +6117,7 @@
         <v>184000</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>72787.92</v>
@@ -6171,7 +6171,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G87" t="n">
         <v>2</v>
@@ -6183,7 +6183,7 @@
         <v>194138.4</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>76798.53</v>
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>4591</v>
+        <v>40</v>
       </c>
       <c r="G88" t="n">
         <v>2</v>
@@ -6249,7 +6249,7 @@
         <v>185000</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>73183.5</v>
@@ -6303,7 +6303,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>5791</v>
+        <v>40</v>
       </c>
       <c r="G89" t="n">
         <v>2</v>
@@ -6315,7 +6315,7 @@
         <v>188000</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>74370.25999999999</v>
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>5184</v>
+        <v>47.09</v>
       </c>
       <c r="G90" t="n">
         <v>2</v>
@@ -6381,7 +6381,7 @@
         <v>189600</v>
       </c>
       <c r="J90" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>75003.2</v>
@@ -6435,7 +6435,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>5832</v>
+        <v>40</v>
       </c>
       <c r="G91" t="n">
         <v>2</v>
@@ -6447,7 +6447,7 @@
         <v>185000</v>
       </c>
       <c r="J91" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>73183.5</v>
@@ -6501,7 +6501,7 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>6596</v>
+        <v>40</v>
       </c>
       <c r="G92" t="n">
         <v>2</v>
@@ -6513,7 +6513,7 @@
         <v>200000</v>
       </c>
       <c r="J92" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>79117.3</v>
@@ -6567,7 +6567,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G93" t="n">
         <v>2</v>
@@ -6579,7 +6579,7 @@
         <v>184100</v>
       </c>
       <c r="J93" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>72827.47</v>
@@ -6633,7 +6633,7 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G94" t="n">
         <v>2</v>
@@ -6645,7 +6645,7 @@
         <v>185000</v>
       </c>
       <c r="J94" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>73183.5</v>
@@ -6699,7 +6699,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>5867</v>
+        <v>40.31</v>
       </c>
       <c r="G95" t="n">
         <v>2</v>
@@ -6711,7 +6711,7 @@
         <v>186000</v>
       </c>
       <c r="J95" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>73579.09</v>
@@ -6765,7 +6765,7 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G96" t="n">
         <v>2</v>
@@ -6777,7 +6777,7 @@
         <v>184100</v>
       </c>
       <c r="J96" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>72827.47</v>
@@ -6831,7 +6831,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G97" t="n">
         <v>2</v>
@@ -6843,7 +6843,7 @@
         <v>190000</v>
       </c>
       <c r="J97" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>75161.42999999999</v>
@@ -6897,7 +6897,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>4618</v>
+        <v>40.31</v>
       </c>
       <c r="G98" t="n">
         <v>2</v>
@@ -6909,7 +6909,7 @@
         <v>200000</v>
       </c>
       <c r="J98" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>79117.3</v>
@@ -6963,7 +6963,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>6322</v>
+        <v>40.31</v>
       </c>
       <c r="G99" t="n">
         <v>2</v>
@@ -6975,7 +6975,7 @@
         <v>184000</v>
       </c>
       <c r="J99" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>72787.92</v>
@@ -7029,7 +7029,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>5867</v>
+        <v>40.31</v>
       </c>
       <c r="G100" t="n">
         <v>2</v>
@@ -7041,7 +7041,7 @@
         <v>200000</v>
       </c>
       <c r="J100" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>79117.3</v>
@@ -7095,7 +7095,7 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>5867</v>
+        <v>40.31</v>
       </c>
       <c r="G101" t="n">
         <v>2</v>
@@ -7107,7 +7107,7 @@
         <v>184000</v>
       </c>
       <c r="J101" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>72787.92</v>
@@ -7161,7 +7161,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>6768</v>
+        <v>40</v>
       </c>
       <c r="G102" t="n">
         <v>2</v>
@@ -7173,7 +7173,7 @@
         <v>187000</v>
       </c>
       <c r="J102" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>73974.67999999999</v>
@@ -7227,7 +7227,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>4620</v>
+        <v>40.31</v>
       </c>
       <c r="G103" t="n">
         <v>2</v>
@@ -7239,7 +7239,7 @@
         <v>210000</v>
       </c>
       <c r="J103" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>83073.16</v>
@@ -7293,7 +7293,7 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>4994</v>
+        <v>43.61</v>
       </c>
       <c r="G104" t="n">
         <v>2</v>
@@ -7305,7 +7305,7 @@
         <v>189000</v>
       </c>
       <c r="J104" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>74765.85000000001</v>
@@ -7359,7 +7359,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G105" t="n">
         <v>2</v>
@@ -7371,7 +7371,7 @@
         <v>184000</v>
       </c>
       <c r="J105" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>72787.92</v>
@@ -7425,7 +7425,7 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>6323</v>
+        <v>40.31</v>
       </c>
       <c r="G106" t="n">
         <v>2</v>
@@ -7437,7 +7437,7 @@
         <v>195000</v>
       </c>
       <c r="J106" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>77139.37</v>
@@ -7491,7 +7491,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G107" t="n">
         <v>2</v>
@@ -7503,7 +7503,7 @@
         <v>205000</v>
       </c>
       <c r="J107" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>81095.23</v>
@@ -7557,7 +7557,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G108" t="n">
         <v>2</v>
@@ -7569,7 +7569,7 @@
         <v>210000</v>
       </c>
       <c r="J108" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>83073.16</v>
@@ -7623,7 +7623,7 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>4000</v>
+        <v>40</v>
       </c>
       <c r="G109" t="n">
         <v>2</v>
@@ -7635,7 +7635,7 @@
         <v>201000</v>
       </c>
       <c r="J109" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>79512.89</v>
@@ -7689,7 +7689,7 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>4031</v>
+        <v>40.31</v>
       </c>
       <c r="G110" t="n">
         <v>2</v>
@@ -7701,7 +7701,7 @@
         <v>202000</v>
       </c>
       <c r="J110" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>79908.47</v>
@@ -7755,7 +7755,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G111" t="n">
         <v>2</v>
@@ -7767,7 +7767,7 @@
         <v>201000</v>
       </c>
       <c r="J111" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>79512.89</v>
@@ -7821,7 +7821,7 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G112" t="n">
         <v>2</v>
@@ -7833,7 +7833,7 @@
         <v>215857.6</v>
       </c>
       <c r="J112" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>85390.35000000001</v>
@@ -7887,7 +7887,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>4994</v>
+        <v>43.61</v>
       </c>
       <c r="G113" t="n">
         <v>2</v>
@@ -7899,7 +7899,7 @@
         <v>200000</v>
       </c>
       <c r="J113" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>79117.3</v>
@@ -7953,7 +7953,7 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>5832</v>
+        <v>40</v>
       </c>
       <c r="G114" t="n">
         <v>2</v>
@@ -7965,7 +7965,7 @@
         <v>187000</v>
       </c>
       <c r="J114" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>73974.67999999999</v>
@@ -8019,7 +8019,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>4617</v>
+        <v>40.31</v>
       </c>
       <c r="G115" t="n">
         <v>2</v>
@@ -8031,7 +8031,7 @@
         <v>187000</v>
       </c>
       <c r="J115" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>73974.67999999999</v>
@@ -8085,7 +8085,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>5836</v>
+        <v>40.31</v>
       </c>
       <c r="G116" t="n">
         <v>2</v>
@@ -8097,7 +8097,7 @@
         <v>190000</v>
       </c>
       <c r="J116" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>75161.42999999999</v>
@@ -8151,7 +8151,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G117" t="n">
         <v>2</v>
@@ -8163,7 +8163,7 @@
         <v>184000</v>
       </c>
       <c r="J117" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>72787.92</v>
@@ -8217,7 +8217,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G118" t="n">
         <v>2</v>
@@ -8229,7 +8229,7 @@
         <v>187000</v>
       </c>
       <c r="J118" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>73974.67999999999</v>
@@ -8283,7 +8283,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>5690</v>
+        <v>40</v>
       </c>
       <c r="G119" t="n">
         <v>2</v>
@@ -8295,7 +8295,7 @@
         <v>209000</v>
       </c>
       <c r="J119" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>82677.58</v>
@@ -8349,7 +8349,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>5004</v>
+        <v>43.61</v>
       </c>
       <c r="G120" t="n">
         <v>2</v>
@@ -8361,7 +8361,7 @@
         <v>197000</v>
       </c>
       <c r="J120" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>77930.53999999999</v>
@@ -8415,7 +8415,7 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>4627</v>
+        <v>40.31</v>
       </c>
       <c r="G121" t="n">
         <v>2</v>
@@ -8427,7 +8427,7 @@
         <v>187118.62</v>
       </c>
       <c r="J121" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>74021.60000000001</v>
@@ -8481,7 +8481,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>4582</v>
+        <v>40</v>
       </c>
       <c r="G122" t="n">
         <v>2</v>
@@ -8493,7 +8493,7 @@
         <v>205500</v>
       </c>
       <c r="J122" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>81293.03</v>
@@ -8547,7 +8547,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>5225</v>
+        <v>43.54</v>
       </c>
       <c r="G123" t="n">
         <v>2</v>
@@ -8559,7 +8559,7 @@
         <v>208550</v>
       </c>
       <c r="J123" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>82499.56</v>
@@ -8613,7 +8613,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>5842</v>
+        <v>49.94</v>
       </c>
       <c r="G124" t="n">
         <v>2</v>
@@ -8625,7 +8625,7 @@
         <v>204000</v>
       </c>
       <c r="J124" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>80699.64999999999</v>
@@ -8679,7 +8679,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>0</v>
+        <v>51.43</v>
       </c>
       <c r="G125" t="n">
         <v>3</v>
@@ -8691,7 +8691,7 @@
         <v>200000</v>
       </c>
       <c r="J125" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>79117.3</v>
@@ -8745,7 +8745,7 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>4365</v>
+        <v>43.65</v>
       </c>
       <c r="G126" t="n">
         <v>2</v>
@@ -8757,7 +8757,7 @@
         <v>195000</v>
       </c>
       <c r="J126" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>77139.37</v>
@@ -8811,7 +8811,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>5845</v>
+        <v>52.86</v>
       </c>
       <c r="G127" t="n">
         <v>3</v>
@@ -8823,7 +8823,7 @@
         <v>210000</v>
       </c>
       <c r="J127" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K127" s="2" t="n">
         <v>83073.16</v>
@@ -8877,7 +8877,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>4538</v>
+        <v>38.4</v>
       </c>
       <c r="G128" t="n">
         <v>2</v>
@@ -8889,7 +8889,7 @@
         <v>216000</v>
       </c>
       <c r="J128" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K128" s="2" t="n">
         <v>85446.67999999999</v>
@@ -8943,7 +8943,7 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>4538</v>
+        <v>38.4</v>
       </c>
       <c r="G129" t="n">
         <v>2</v>
@@ -8955,7 +8955,7 @@
         <v>232000</v>
       </c>
       <c r="J129" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K129" s="2" t="n">
         <v>91776.07000000001</v>
@@ -9009,7 +9009,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>0</v>
+        <v>57.99</v>
       </c>
       <c r="G130" t="n">
         <v>2</v>
@@ -9021,7 +9021,7 @@
         <v>235000</v>
       </c>
       <c r="J130" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K130" s="2" t="n">
         <v>92962.83</v>
@@ -9075,7 +9075,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>5150</v>
+        <v>38.4</v>
       </c>
       <c r="G131" t="n">
         <v>1</v>
@@ -9087,7 +9087,7 @@
         <v>200000</v>
       </c>
       <c r="J131" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K131" s="2" t="n">
         <v>79117.3</v>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>7621</v>
+        <v>38.4</v>
       </c>
       <c r="G132" t="n">
         <v>2</v>
@@ -9153,7 +9153,7 @@
         <v>204202.99</v>
       </c>
       <c r="J132" s="3" t="n">
-        <v>3956</v>
+        <v>39.56</v>
       </c>
       <c r="K132" s="2" t="n">
         <v>80779.95</v>
@@ -9207,7 +9207,7 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>0</v>
+        <v>3328.92</v>
       </c>
       <c r="H133" s="2" t="n">
         <v>520685.78</v>
@@ -9216,7 +9216,7 @@
         <v>860000</v>
       </c>
       <c r="J133" s="3" t="n">
-        <v>3946</v>
+        <v>39.46</v>
       </c>
       <c r="K133" s="2" t="n">
         <v>339314.22</v>
@@ -9270,7 +9270,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>4002</v>
+        <v>36.4</v>
       </c>
       <c r="G134" t="n">
         <v>2</v>
@@ -9282,7 +9282,7 @@
         <v>148000</v>
       </c>
       <c r="J134" s="3" t="n">
-        <v>3896</v>
+        <v>38.96</v>
       </c>
       <c r="K134" s="2" t="n">
         <v>57650.03</v>
@@ -9336,7 +9336,7 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>5270</v>
+        <v>46.68</v>
       </c>
       <c r="G135" t="n">
         <v>2</v>
@@ -9348,7 +9348,7 @@
         <v>305500</v>
       </c>
       <c r="J135" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K135" s="2" t="n">
         <v>118440.98</v>
@@ -9402,7 +9402,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>7239</v>
+        <v>61.95</v>
       </c>
       <c r="G136" t="n">
         <v>2</v>
@@ -9414,7 +9414,7 @@
         <v>251000</v>
       </c>
       <c r="J136" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K136" s="2" t="n">
         <v>97311.57000000001</v>
@@ -9468,7 +9468,7 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>4915</v>
+        <v>41.6</v>
       </c>
       <c r="G137" t="n">
         <v>2</v>
@@ -9480,7 +9480,7 @@
         <v>270000</v>
       </c>
       <c r="J137" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K137" s="2" t="n">
         <v>104677.78</v>
@@ -9534,7 +9534,7 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>5943</v>
+        <v>48.13</v>
       </c>
       <c r="G138" t="n">
         <v>2</v>
@@ -9546,7 +9546,7 @@
         <v>280000</v>
       </c>
       <c r="J138" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K138" s="2" t="n">
         <v>108554.74</v>
@@ -9600,7 +9600,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>4200</v>
+        <v>42</v>
       </c>
       <c r="G139" t="n">
         <v>2</v>
@@ -9612,7 +9612,7 @@
         <v>240000</v>
       </c>
       <c r="J139" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K139" s="2" t="n">
         <v>93046.92</v>
@@ -9666,7 +9666,7 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>4200</v>
+        <v>42</v>
       </c>
       <c r="G140" t="n">
         <v>2</v>
@@ -9678,7 +9678,7 @@
         <v>240000</v>
       </c>
       <c r="J140" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K140" s="2" t="n">
         <v>93046.92</v>
@@ -9732,7 +9732,7 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>4200</v>
+        <v>42</v>
       </c>
       <c r="G141" t="n">
         <v>2</v>
@@ -9744,7 +9744,7 @@
         <v>240000</v>
       </c>
       <c r="J141" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K141" s="2" t="n">
         <v>93046.92</v>
@@ -9798,7 +9798,7 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="H142" s="2" t="n">
         <v>144503.86</v>
@@ -9807,7 +9807,7 @@
         <v>236000</v>
       </c>
       <c r="J142" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K142" s="2" t="n">
         <v>91496.14</v>
@@ -9861,7 +9861,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>6055</v>
+        <v>55.26</v>
       </c>
       <c r="G143" t="n">
         <v>2</v>
@@ -9873,7 +9873,7 @@
         <v>271500</v>
       </c>
       <c r="J143" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K143" s="2" t="n">
         <v>105259.33</v>
@@ -9927,7 +9927,7 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>6024</v>
+        <v>52.6</v>
       </c>
       <c r="G144" t="n">
         <v>2</v>
@@ -9939,7 +9939,7 @@
         <v>236000</v>
       </c>
       <c r="J144" s="3" t="n">
-        <v>3877</v>
+        <v>38.77</v>
       </c>
       <c r="K144" s="2" t="n">
         <v>91496.14</v>
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>3977</v>
+        <v>38.6</v>
       </c>
       <c r="G145" t="n">
         <v>2</v>
@@ -10005,7 +10005,7 @@
         <v>167000</v>
       </c>
       <c r="J145" s="3" t="n">
-        <v>3824</v>
+        <v>38.24</v>
       </c>
       <c r="K145" s="2" t="n">
         <v>63860.07</v>
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>4588</v>
+        <v>40.31</v>
       </c>
       <c r="G146" t="n">
         <v>2</v>
@@ -10071,7 +10071,7 @@
         <v>184000</v>
       </c>
       <c r="J146" s="3" t="n">
-        <v>3706</v>
+        <v>37.06</v>
       </c>
       <c r="K146" s="2" t="n">
         <v>68186.11</v>
@@ -10125,7 +10125,7 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>5010</v>
+        <v>50.1</v>
       </c>
       <c r="G147" t="n">
         <v>2</v>
@@ -10137,7 +10137,7 @@
         <v>189000</v>
       </c>
       <c r="J147" s="3" t="n">
-        <v>3706</v>
+        <v>37.06</v>
       </c>
       <c r="K147" s="2" t="n">
         <v>70039</v>
@@ -10191,7 +10191,7 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G148" t="n">
         <v>2</v>
@@ -10203,7 +10203,7 @@
         <v>190000</v>
       </c>
       <c r="J148" s="3" t="n">
-        <v>3706</v>
+        <v>37.06</v>
       </c>
       <c r="K148" s="2" t="n">
         <v>70409.57000000001</v>
@@ -10257,7 +10257,7 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>6398</v>
+        <v>55.06</v>
       </c>
       <c r="G149" t="n">
         <v>2</v>
@@ -10269,7 +10269,7 @@
         <v>204000</v>
       </c>
       <c r="J149" s="3" t="n">
-        <v>3706</v>
+        <v>37.06</v>
       </c>
       <c r="K149" s="2" t="n">
         <v>75597.64999999999</v>
@@ -10323,7 +10323,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>4495</v>
+        <v>40.01</v>
       </c>
       <c r="G150" t="n">
         <v>2</v>
@@ -10335,7 +10335,7 @@
         <v>190000</v>
       </c>
       <c r="J150" s="3" t="n">
-        <v>3706</v>
+        <v>37.06</v>
       </c>
       <c r="K150" s="2" t="n">
         <v>70409.57000000001</v>
@@ -10389,7 +10389,7 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>4930</v>
+        <v>42.57</v>
       </c>
       <c r="G151" t="n">
         <v>2</v>
@@ -10401,7 +10401,7 @@
         <v>198363.85</v>
       </c>
       <c r="J151" s="3" t="n">
-        <v>3706</v>
+        <v>37.06</v>
       </c>
       <c r="K151" s="2" t="n">
         <v>73509.02</v>
@@ -10455,7 +10455,7 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>0</v>
+        <v>53.29</v>
       </c>
       <c r="G152" t="n">
         <v>2</v>
@@ -10467,7 +10467,7 @@
         <v>217000</v>
       </c>
       <c r="J152" s="3" t="n">
-        <v>3706</v>
+        <v>37.06</v>
       </c>
       <c r="K152" s="2" t="n">
         <v>80415.14</v>
@@ -10521,7 +10521,7 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>6264</v>
+        <v>54.99</v>
       </c>
       <c r="G153" t="n">
         <v>2</v>
@@ -10533,7 +10533,7 @@
         <v>240000</v>
       </c>
       <c r="J153" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K153" s="2" t="n">
         <v>87044.57000000001</v>
@@ -10587,7 +10587,7 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>0</v>
+        <v>547.75</v>
       </c>
       <c r="G154" t="n">
         <v>5</v>
@@ -10599,7 +10599,7 @@
         <v>3800000</v>
       </c>
       <c r="J154" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K154" s="2" t="n">
         <v>1378205.66</v>
@@ -10653,7 +10653,7 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>9099</v>
+        <v>90.98999999999999</v>
       </c>
       <c r="G155" t="n">
         <v>3</v>
@@ -10665,7 +10665,7 @@
         <v>370000</v>
       </c>
       <c r="J155" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K155" s="2" t="n">
         <v>134193.71</v>
@@ -10719,7 +10719,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>9825</v>
+        <v>87.59</v>
       </c>
       <c r="G156" t="n">
         <v>3</v>
@@ -10731,7 +10731,7 @@
         <v>415000</v>
       </c>
       <c r="J156" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K156" s="2" t="n">
         <v>150514.57</v>
@@ -10785,7 +10785,7 @@
         </is>
       </c>
       <c r="F157" t="n">
-        <v>5970</v>
+        <v>59.7</v>
       </c>
       <c r="G157" t="n">
         <v>2</v>
@@ -10797,7 +10797,7 @@
         <v>282000</v>
       </c>
       <c r="J157" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K157" s="2" t="n">
         <v>102277.37</v>
@@ -10851,7 +10851,7 @@
         </is>
       </c>
       <c r="F158" t="n">
-        <v>41032</v>
+        <v>410.32</v>
       </c>
       <c r="G158" t="n">
         <v>3</v>
@@ -10863,7 +10863,7 @@
         <v>2280000</v>
       </c>
       <c r="J158" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K158" s="2" t="n">
         <v>826923.4</v>
@@ -10917,7 +10917,7 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>13891</v>
+        <v>51.72</v>
       </c>
       <c r="G159" t="n">
         <v>4</v>
@@ -10929,7 +10929,7 @@
         <v>390000</v>
       </c>
       <c r="J159" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K159" s="2" t="n">
         <v>141447.42</v>
@@ -10983,7 +10983,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>0</v>
+        <v>70.06999999999999</v>
       </c>
       <c r="H160" s="2" t="n">
         <v>235806.29</v>
@@ -10992,7 +10992,7 @@
         <v>370000</v>
       </c>
       <c r="J160" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K160" s="2" t="n">
         <v>134193.71</v>
@@ -11046,7 +11046,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="H161" s="2" t="n">
         <v>184821.15</v>
@@ -11055,7 +11055,7 @@
         <v>290000</v>
       </c>
       <c r="J161" s="3" t="n">
-        <v>3627</v>
+        <v>36.27</v>
       </c>
       <c r="K161" s="2" t="n">
         <v>105178.85</v>
@@ -11109,7 +11109,7 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G162" t="n">
         <v>3</v>
@@ -11121,7 +11121,7 @@
         <v>290000</v>
       </c>
       <c r="J162" s="3" t="n">
-        <v>3545</v>
+        <v>35.45</v>
       </c>
       <c r="K162" s="2" t="n">
         <v>102777.04</v>
@@ -11175,7 +11175,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>12/07/2026 às 22:57</t>
+          <t>12/07/2026 às 23:06</t>
         </is>
       </c>
     </row>
@@ -11206,7 +11206,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4019.9</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 15:35 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Imóveis'!$A$1:$P$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Imóveis'!$A$1:$R$162</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P162"/>
+  <dimension ref="A1:R162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -455,7 +455,9 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,6 +538,16 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Edital (PDF)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Matrícula (PDF)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>Descrição</t>
         </is>
       </c>
@@ -597,7 +609,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=10139954</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010139954.pdf</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Gleba, 0.00 de área total, 0.00 de área privativa, 72600.00 de área do terreno.</t>
         </is>
@@ -662,6 +680,16 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010011968.pdf</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
           <t>Comercial, 0.00 de área total, 2890.80 de área privativa, 3960.00 de área do terreno.</t>
         </is>
       </c>
@@ -728,6 +756,16 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444419331060.pdf</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 61.60 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), 1 lavabo(s), cozinha.</t>
         </is>
       </c>
@@ -794,6 +832,16 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787706961580.pdf</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -858,7 +906,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704108538</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704108538.pdf</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>Apartamento, 45.90 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -924,7 +978,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705420250</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705420250.pdf</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>Apartamento, 101.65 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -992,6 +1052,16 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705008413.pdf</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 47.15 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1056,7 +1126,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703998130</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703998130.pdf</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
         <is>
           <t>Apartamento, 40.31 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -1122,7 +1198,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703714736</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703714736.pdf</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -1190,6 +1272,16 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555516351888.pdf</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 42.27 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1256,6 +1348,16 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787708753594.pdf</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
           <t>Apartamento, 43.37 de área total, 41.54 de área privativa, 0.00 de área do terreno,  2 qto(s), 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1320,7 +1422,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703152487</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703152487.pdf</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -1388,6 +1496,16 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444418135747.pdf</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 50.17 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1452,7 +1570,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444421418659</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444421418659.pdf</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
         <is>
           <t>Casa, 433.88 de área total, 433.88 de área privativa, 780.00 de área do terreno,  5 qto(s), a.serv, WC, 4 sala(s), 1 lavabo(s), cozinha.</t>
         </is>
@@ -1520,6 +1644,16 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444407507011.pdf</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
           <t>Casa, 0.00 de área total, 86.93 de área privativa, 177.08 de área do terreno,  3 qto(s), WC, 2 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1586,6 +1720,16 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444433866030.pdf</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
           <t>Apartamento, 49.30 de área total, 42.57 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1652,6 +1796,16 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787708379374.pdf</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
           <t>Apartamento, 54.62 de área total, 41.54 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1718,6 +1872,16 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787709302057.pdf</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
           <t>Apartamento, 43.37 de área total, 41.54 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1782,7 +1946,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787708373384</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787708373384.pdf</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
         <is>
           <t>Apartamento, 54.62 de área total, 41.54 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -1850,6 +2020,16 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555528701382.pdf</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
           <t>Apartamento, 45.00 de área total, 43.12 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1916,6 +2096,16 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555533721264.pdf</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
           <t>Apartamento, 40.52 de área total, 37.80 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, Terraco, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -1982,6 +2172,16 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787711689621.pdf</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
           <t>Apartamento, 42.28 de área total, 41.70 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -2046,7 +2246,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787701930377</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701930377.pdf</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
         <is>
           <t>Apartamento, 50.03 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2114,6 +2320,16 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702314505.pdf</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -2178,7 +2394,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702327518</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702327518.pdf</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2244,7 +2466,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702406663</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702406663.pdf</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
         <is>
           <t>Apartamento, 4019.21 de área total, 40.13 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2310,7 +2538,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702413406</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702413406.pdf</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
         <is>
           <t>Apartamento, 45.92 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2376,7 +2610,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702492527</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702492527.pdf</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
         <is>
           <t>Apartamento, 52.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2442,7 +2682,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702551558</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702551558.pdf</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2510,6 +2756,16 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702693310.pdf</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -2576,6 +2832,16 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702831976.pdf</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -2640,7 +2906,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703271915</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703271915.pdf</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2706,7 +2978,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703275635</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703275635.pdf</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
         <is>
           <t>Apartamento, 52.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2772,7 +3050,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703305208</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703305208.pdf</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2840,6 +3124,16 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703484536.pdf</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -2904,7 +3198,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703539160</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703539160.pdf</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
         <is>
           <t>Apartamento, 46.26 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 2 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -2970,7 +3270,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703661217</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703661217.pdf</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 52.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3036,7 +3342,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703670038</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703670038.pdf</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
         <is>
           <t>Apartamento, 50.03 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3102,7 +3414,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787706657300</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787706657300.pdf</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
         <is>
           <t>Apartamento, 52.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3168,7 +3486,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787706692334</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787706692334.pdf</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3234,7 +3558,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710716757</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710716757.pdf</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3302,6 +3632,16 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444428790721.pdf</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
           <t>Apartamento, 44.90 de área total, 40.10 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -3366,7 +3706,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704480631</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704480631.pdf</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
         <is>
           <t>Apartamento, 45.87 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3434,6 +3780,16 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704497119.pdf</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
           <t>Apartamento, 50.08 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -3498,7 +3854,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704497666</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704497666.pdf</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
         <is>
           <t>Apartamento, 47.38 de área total, 41.51 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3564,7 +3926,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704497801</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704497801.pdf</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3630,7 +3998,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704800784</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704800784.pdf</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
         <is>
           <t>Apartamento, 102.33 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3696,7 +4070,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704962300</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704962300.pdf</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3762,7 +4142,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705007468</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705007468.pdf</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3828,7 +4214,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705163931</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705163931.pdf</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3894,7 +4286,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705172213</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705172213.pdf</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
         <is>
           <t>Apartamento, 58.32 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -3960,7 +4358,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705192680</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705192680.pdf</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
         <is>
           <t>Apartamento, 45.87 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4026,7 +4430,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705273168</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr">
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705273168.pdf</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4092,7 +4502,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705286154</t>
         </is>
       </c>
-      <c r="P55" t="inlineStr">
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705286154.pdf</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
         <is>
           <t>Apartamento, 46.20 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, Terraco, 1 vaga(s) de garagem.</t>
         </is>
@@ -4158,7 +4574,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705371763</t>
         </is>
       </c>
-      <c r="P56" t="inlineStr">
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705371763.pdf</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
         <is>
           <t>Apartamento, 47.59 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4224,7 +4646,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705411382</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr">
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705411382.pdf</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4290,7 +4718,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705470630</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr">
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705470630.pdf</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4356,7 +4790,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787706024617</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr">
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787706024617.pdf</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4422,7 +4862,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787709582823</t>
         </is>
       </c>
-      <c r="P60" t="inlineStr">
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787709582823.pdf</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4490,6 +4936,16 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787709839662.pdf</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -4554,7 +5010,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710470111</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr">
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710470111.pdf</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
         <is>
           <t>Apartamento, 46.20 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4620,7 +5082,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710517002</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr">
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710517002.pdf</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
         <is>
           <t>Apartamento, 45.87 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4686,7 +5154,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710659753</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr">
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710659753.pdf</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
         <is>
           <t>Apartamento, 45.87 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4752,7 +5226,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710915423</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr">
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710915423.pdf</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
         <is>
           <t>Apartamento, 45.87 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4818,7 +5298,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703697718</t>
         </is>
       </c>
-      <c r="P66" t="inlineStr">
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703697718.pdf</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
         <is>
           <t>Apartamento, 637.60 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4884,7 +5370,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703952092</t>
         </is>
       </c>
-      <c r="P67" t="inlineStr">
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703952092.pdf</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -4950,7 +5442,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705586328</t>
         </is>
       </c>
-      <c r="P68" t="inlineStr">
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705586328.pdf</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
         <is>
           <t>Apartamento, 46.34 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -5018,6 +5516,16 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555536055583.pdf</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
           <t>Apartamento, 49.88 de área total, 43.51 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -5082,7 +5590,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714493566</t>
         </is>
       </c>
-      <c r="P70" t="inlineStr">
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714493566.pdf</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
         <is>
           <t>Apartamento, 58.30 de área total, 49.84 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -5148,7 +5662,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555512847072</t>
         </is>
       </c>
-      <c r="P71" t="inlineStr">
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555512847072.pdf</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 35.10 de área privativa, 155.49 de área do terreno,  1 qto(s), WC, 1 sala(s), cozinha.</t>
         </is>
@@ -5214,7 +5734,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555515362061</t>
         </is>
       </c>
-      <c r="P72" t="inlineStr">
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555515362061.pdf</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
         <is>
           <t>Casa, 47.30 de área total, 47.30 de área privativa, 127.91 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
         </is>
@@ -5282,6 +5808,16 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715025965.pdf</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
           <t>Apartamento, 101.20 de área total, 38.68 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -5346,7 +5882,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702208306</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr">
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702208306.pdf</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -5412,7 +5954,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787707492428</t>
         </is>
       </c>
-      <c r="P75" t="inlineStr">
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787707492428.pdf</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
         <is>
           <t>Apartamento, 42.12 de área total, 40.32 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -5480,6 +6028,16 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787713103853.pdf</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
           <t>Apartamento, 58.17 de área total, 41.11 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -5546,6 +6104,16 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714502816.pdf</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
           <t>Apartamento, 45.67 de área total, 41.11 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -5612,6 +6180,16 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787711125159.pdf</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
           <t>Apartamento, 50.16 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, Terraco, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -5678,6 +6256,16 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703438488.pdf</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
           <t>Apartamento, 45.49 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -5744,6 +6332,16 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555532121042.pdf</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
           <t>Apartamento, 44.57 de área total, 41.70 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -5808,7 +6406,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787701698989</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701698989.pdf</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -5876,6 +6480,16 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701904252.pdf</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
           <t>Apartamento, 50.04 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -5940,7 +6554,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702328662</t>
         </is>
       </c>
-      <c r="P83" t="inlineStr">
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702328662.pdf</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
         <is>
           <t>Apartamento, 62.82 de área total, 44.83 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6006,7 +6626,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703061902</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr">
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703061902.pdf</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
         <is>
           <t>Apartamento, 46.26 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6072,7 +6698,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703300125</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr">
+      <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703300125.pdf</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
         <is>
           <t>Apartamento, 50.04 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6138,7 +6770,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703620065</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr">
+      <c r="P86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703620065.pdf</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6204,7 +6842,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704032140</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr">
+      <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704032140.pdf</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6270,7 +6914,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705513541</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr">
+      <c r="P88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705513541.pdf</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6336,7 +6986,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705920686</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr">
+      <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705920686.pdf</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
         <is>
           <t>Apartamento, 57.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6404,6 +7060,16 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787708326874.pdf</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
           <t>Apartamento, 51.84 de área total, 47.09 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -6468,7 +7134,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444433965534</t>
         </is>
       </c>
-      <c r="P91" t="inlineStr">
+      <c r="P91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444433965534.pdf</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
         <is>
           <t>Apartamento, 58.32 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6536,6 +7208,16 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704497623.pdf</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
           <t>Apartamento, 65.96 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, Terraco, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -6600,7 +7282,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704512177</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr">
+      <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704512177.pdf</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6666,7 +7354,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704848876</t>
         </is>
       </c>
-      <c r="P94" t="inlineStr">
+      <c r="P94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704848876.pdf</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6732,7 +7426,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704880206</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr">
+      <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704880206.pdf</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
         <is>
           <t>Apartamento, 58.67 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6798,7 +7498,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704882381</t>
         </is>
       </c>
-      <c r="P96" t="inlineStr">
+      <c r="P96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704882381.pdf</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6864,7 +7570,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704947556</t>
         </is>
       </c>
-      <c r="P97" t="inlineStr">
+      <c r="P97" t="inlineStr"/>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704947556.pdf</t>
+        </is>
+      </c>
+      <c r="R97" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6930,7 +7642,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787704995690</t>
         </is>
       </c>
-      <c r="P98" t="inlineStr">
+      <c r="P98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787704995690.pdf</t>
+        </is>
+      </c>
+      <c r="R98" t="inlineStr">
         <is>
           <t>Apartamento, 46.18 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -6996,7 +7714,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705182766</t>
         </is>
       </c>
-      <c r="P99" t="inlineStr">
+      <c r="P99" t="inlineStr"/>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705182766.pdf</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
         <is>
           <t>Apartamento, 63.22 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7062,7 +7786,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705222474</t>
         </is>
       </c>
-      <c r="P100" t="inlineStr">
+      <c r="P100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705222474.pdf</t>
+        </is>
+      </c>
+      <c r="R100" t="inlineStr">
         <is>
           <t>Apartamento, 58.67 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7128,7 +7858,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705231058</t>
         </is>
       </c>
-      <c r="P101" t="inlineStr">
+      <c r="P101" t="inlineStr"/>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705231058.pdf</t>
+        </is>
+      </c>
+      <c r="R101" t="inlineStr">
         <is>
           <t>Apartamento, 58.67 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7194,7 +7930,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705242742</t>
         </is>
       </c>
-      <c r="P102" t="inlineStr">
+      <c r="P102" t="inlineStr"/>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705242742.pdf</t>
+        </is>
+      </c>
+      <c r="R102" t="inlineStr">
         <is>
           <t>Apartamento, 67.68 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, Terraco, 1 vaga(s) de garagem.</t>
         </is>
@@ -7260,7 +8002,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705253957</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr">
+      <c r="P103" t="inlineStr"/>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705253957.pdf</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
         <is>
           <t>Apartamento, 46.20 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7326,7 +8074,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705273699</t>
         </is>
       </c>
-      <c r="P104" t="inlineStr">
+      <c r="P104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705273699.pdf</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
         <is>
           <t>Apartamento, 49.94 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7392,7 +8146,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705326180</t>
         </is>
       </c>
-      <c r="P105" t="inlineStr">
+      <c r="P105" t="inlineStr"/>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705326180.pdf</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7458,7 +8218,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705391900</t>
         </is>
       </c>
-      <c r="P106" t="inlineStr">
+      <c r="P106" t="inlineStr"/>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705391900.pdf</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
         <is>
           <t>Apartamento, 63.23 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, Terraco, 1 vaga(s) de garagem.</t>
         </is>
@@ -7524,7 +8290,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705475852</t>
         </is>
       </c>
-      <c r="P107" t="inlineStr">
+      <c r="P107" t="inlineStr"/>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705475852.pdf</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7590,7 +8362,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705477146</t>
         </is>
       </c>
-      <c r="P108" t="inlineStr">
+      <c r="P108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705477146.pdf</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7658,6 +8436,16 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705624556.pdf</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
           <t>Apartamento, 40.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -7724,6 +8512,16 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705639308.pdf</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
           <t>Apartamento, 40.31 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -7790,6 +8588,16 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705647980.pdf</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -7854,7 +8662,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705691571</t>
         </is>
       </c>
-      <c r="P112" t="inlineStr">
+      <c r="P112" t="inlineStr"/>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705691571.pdf</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -7922,6 +8736,16 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705717481.pdf</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
           <t>Apartamento, 49.94 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -7986,7 +8810,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705962249</t>
         </is>
       </c>
-      <c r="P114" t="inlineStr">
+      <c r="P114" t="inlineStr"/>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705962249.pdf</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
         <is>
           <t>Apartamento, 58.32 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8052,7 +8882,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710324760</t>
         </is>
       </c>
-      <c r="P115" t="inlineStr">
+      <c r="P115" t="inlineStr"/>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710324760.pdf</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
         <is>
           <t>Apartamento, 46.17 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8118,7 +8954,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710357293</t>
         </is>
       </c>
-      <c r="P116" t="inlineStr">
+      <c r="P116" t="inlineStr"/>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710357293.pdf</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
         <is>
           <t>Apartamento, 58.36 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8184,7 +9026,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710694770</t>
         </is>
       </c>
-      <c r="P117" t="inlineStr">
+      <c r="P117" t="inlineStr"/>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710694770.pdf</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8250,7 +9098,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702149954</t>
         </is>
       </c>
-      <c r="P118" t="inlineStr">
+      <c r="P118" t="inlineStr"/>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702149954.pdf</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8316,7 +9170,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787702847805</t>
         </is>
       </c>
-      <c r="P119" t="inlineStr">
+      <c r="P119" t="inlineStr"/>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702847805.pdf</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
         <is>
           <t>Apartamento, 56.90 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8382,7 +9242,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703188899</t>
         </is>
       </c>
-      <c r="P120" t="inlineStr">
+      <c r="P120" t="inlineStr"/>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703188899.pdf</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
         <is>
           <t>Apartamento, 50.04 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8448,7 +9314,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703202964</t>
         </is>
       </c>
-      <c r="P121" t="inlineStr">
+      <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703202964.pdf</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8514,7 +9386,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787709676569</t>
         </is>
       </c>
-      <c r="P122" t="inlineStr">
+      <c r="P122" t="inlineStr"/>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787709676569.pdf</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8582,6 +9460,16 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787700995319.pdf</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr">
+        <is>
           <t>Apartamento, 52.25 de área total, 43.54 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -8646,7 +9534,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787710407215</t>
         </is>
       </c>
-      <c r="P124" t="inlineStr">
+      <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710407215.pdf</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
         <is>
           <t>Apartamento, 58.42 de área total, 49.94 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -8712,7 +9606,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444404798498</t>
         </is>
       </c>
-      <c r="P125" t="inlineStr">
+      <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404798498.pdf</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 51.43 de área privativa, 0.00 de área do terreno,  3 qto(s), 1 sala(s), cozinha.</t>
         </is>
@@ -8778,7 +9678,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444406189855</t>
         </is>
       </c>
-      <c r="P126" t="inlineStr">
+      <c r="P126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444406189855.pdf</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
         <is>
           <t>Casa, 43.65 de área total, 43.65 de área privativa, 71.60 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
         </is>
@@ -8846,6 +9752,16 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705100042.pdf</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
           <t>Apartamento, 58.45 de área total, 52.86 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -8912,6 +9828,16 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787712957700.pdf</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
           <t>Apartamento, 45.38 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), 1 sala(s), 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -8978,6 +9904,16 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715863944.pdf</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
           <t>Apartamento, 45.38 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9044,6 +9980,16 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444422964744.pdf</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 57.99 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9110,6 +10056,16 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703103958.pdf</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr">
+        <is>
           <t>Apartamento, 51.50 de área total, 38.40 de área privativa, 0.00 de área do terreno,  1 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9176,6 +10132,16 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715235463.pdf</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
           <t>Apartamento, 76.21 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9237,7 +10203,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444422825932</t>
         </is>
       </c>
-      <c r="P133" t="inlineStr">
+      <c r="P133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444422825932.pdf</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
         <is>
           <t>Terreno, 0.00 de área total, 0.00 de área privativa, 3328.92 de área do terreno.</t>
         </is>
@@ -9305,6 +10277,16 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444422580050.pdf</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
           <t>Apartamento, 40.02 de área total, 36.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -9371,6 +10353,16 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715190850.pdf</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
           <t>Apartamento, 52.70 de área total, 46.68 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9437,6 +10429,16 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716620441.pdf</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
           <t>Apartamento, 72.39 de área total, 61.95 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9503,6 +10505,16 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715858002.pdf</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
           <t>Apartamento, 49.15 de área total, 41.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9569,6 +10581,16 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444430740965.pdf</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
           <t>Apartamento, 59.43 de área total, 48.13 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -9635,6 +10657,16 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787712390409.pdf</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -9701,6 +10733,16 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714019724.pdf</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -9767,6 +10809,16 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714335693.pdf</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -9830,6 +10882,16 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716737225.pdf</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
           <t>Casa, 0.00 de área total, 42.00 de área privativa, 78.00 de área do terreno.</t>
         </is>
       </c>
@@ -9896,6 +10958,16 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787718250838.pdf</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
           <t>Apartamento, 60.55 de área total, 55.26 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -9962,6 +11034,16 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555532572478.pdf</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
           <t>Apartamento, 60.24 de área total, 52.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10028,6 +11110,16 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444417159547.pdf</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
           <t>Casa, 39.77 de área total, 38.60 de área privativa, 108.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10094,6 +11186,16 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1787700557135.pdf</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
           <t>Apartamento, 45.88 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10160,6 +11262,16 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518325604.pdf</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
           <t>Casa, 50.10 de área total, 50.10 de área privativa, 69.70 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -10224,7 +11336,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787701955078</t>
         </is>
       </c>
-      <c r="P148" t="inlineStr">
+      <c r="P148" t="inlineStr"/>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701955078.pdf</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -10292,6 +11410,16 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414235560.pdf</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
           <t>Apartamento, 63.98 de área total, 55.06 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10358,6 +11486,16 @@
       </c>
       <c r="P150" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518647563.pdf</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
           <t>Apartamento, 44.95 de área total, 40.01 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
@@ -10424,6 +11562,16 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423636724.pdf</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
           <t>Apartamento, 49.30 de área total, 42.57 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10490,6 +11638,16 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444424287210.pdf</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
           <t>Apartamento, 0.00 de área total, 53.29 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10556,6 +11714,16 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555533967557.pdf</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
           <t>Apartamento, 62.64 de área total, 54.99 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10620,7 +11788,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=10284141</t>
         </is>
       </c>
-      <c r="P154" t="inlineStr">
+      <c r="P154" t="inlineStr"/>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010284141.pdf</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 547.75 de área privativa, 1468.00 de área do terreno,  5 qto(s), varanda, a.serv, WC, WC Emp, 2 sala(s), 1 lavabo(s), cozinha, Terraco.</t>
         </is>
@@ -10688,6 +11862,16 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444407173466.pdf</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
           <t>Casa, 90.99 de área total, 90.99 de área privativa, 74.81 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), 1 lavabo(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10754,6 +11938,16 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1065020080212.pdf</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
           <t>Apartamento, 98.25 de área total, 87.59 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, WC Emp, 1 sala(s), DCE, cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10820,6 +12014,16 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404619259.pdf</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
           <t>Apartamento, 59.70 de área total, 59.70 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
       </c>
@@ -10884,7 +12088,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1555528553075</t>
         </is>
       </c>
-      <c r="P158" t="inlineStr">
+      <c r="P158" t="inlineStr"/>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1555528553075.pdf</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
         <is>
           <t>Casa, 410.32 de área total, 410.32 de área privativa, 528.00 de área do terreno,  3 qto(s), a.serv, WC, 4 sala(s), cozinha.</t>
         </is>
@@ -10950,7 +12160,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444418870180</t>
         </is>
       </c>
-      <c r="P159" t="inlineStr">
+      <c r="P159" t="inlineStr"/>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418870180.pdf</t>
+        </is>
+      </c>
+      <c r="R159" t="inlineStr">
         <is>
           <t>Casa, 138.91 de área total, 51.72 de área privativa, 194.79 de área do terreno,  4 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
         </is>
@@ -11015,6 +12231,16 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010286302.pdf</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
           <t>Casa, 0.00 de área total, 70.07 de área privativa, 207.66 de área do terreno.</t>
         </is>
       </c>
@@ -11076,7 +12302,13 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444418887481</t>
         </is>
       </c>
-      <c r="P161" t="inlineStr">
+      <c r="P161" t="inlineStr"/>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418887481.pdf</t>
+        </is>
+      </c>
+      <c r="R161" t="inlineStr">
         <is>
           <t>Terreno, 0.00 de área total, 0.00 de área privativa, 480.00 de área do terreno.</t>
         </is>
@@ -11144,12 +12376,22 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423249372.pdf</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
           <t>Casa, 0.00 de área total, 60.00 de área privativa, 120.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P162"/>
+  <autoFilter ref="A1:R162"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11175,7 +12417,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 09:35</t>
+          <t>13/07/2026 às 12:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 15:43 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Terreno</t>
+          <t>Gleba</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -644,7 +644,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Terreno</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -12417,7 +12417,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 12:35</t>
+          <t>13/07/2026 às 12:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 16:10 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -10503,16 +10503,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715858002</t>
         </is>
       </c>
-      <c r="P137" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q137" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715858002.pdf</t>
-        </is>
-      </c>
+      <c r="P137" t="inlineStr"/>
+      <c r="Q137" t="inlineStr"/>
       <c r="R137" t="inlineStr">
         <is>
           <t>Apartamento, 49.15 de área total, 41.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10579,16 +10571,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444430740965</t>
         </is>
       </c>
-      <c r="P138" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q138" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444430740965.pdf</t>
-        </is>
-      </c>
+      <c r="P138" t="inlineStr"/>
+      <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr">
         <is>
           <t>Apartamento, 59.43 de área total, 48.13 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10655,16 +10639,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787712390409</t>
         </is>
       </c>
-      <c r="P139" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q139" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787712390409.pdf</t>
-        </is>
-      </c>
+      <c r="P139" t="inlineStr"/>
+      <c r="Q139" t="inlineStr"/>
       <c r="R139" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10731,16 +10707,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714019724</t>
         </is>
       </c>
-      <c r="P140" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q140" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714019724.pdf</t>
-        </is>
-      </c>
+      <c r="P140" t="inlineStr"/>
+      <c r="Q140" t="inlineStr"/>
       <c r="R140" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10807,16 +10775,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714335693</t>
         </is>
       </c>
-      <c r="P141" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q141" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714335693.pdf</t>
-        </is>
-      </c>
+      <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr"/>
       <c r="R141" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10880,16 +10840,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716737225</t>
         </is>
       </c>
-      <c r="P142" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q142" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716737225.pdf</t>
-        </is>
-      </c>
+      <c r="P142" t="inlineStr"/>
+      <c r="Q142" t="inlineStr"/>
       <c r="R142" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 42.00 de área privativa, 78.00 de área do terreno.</t>
@@ -10956,16 +10908,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787718250838</t>
         </is>
       </c>
-      <c r="P143" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q143" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787718250838.pdf</t>
-        </is>
-      </c>
+      <c r="P143" t="inlineStr"/>
+      <c r="Q143" t="inlineStr"/>
       <c r="R143" t="inlineStr">
         <is>
           <t>Apartamento, 60.55 de área total, 55.26 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11032,16 +10976,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555532572478</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q144" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555532572478.pdf</t>
-        </is>
-      </c>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
       <c r="R144" t="inlineStr">
         <is>
           <t>Apartamento, 60.24 de área total, 52.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11108,16 +11044,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444417159547</t>
         </is>
       </c>
-      <c r="P145" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q145" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444417159547.pdf</t>
-        </is>
-      </c>
+      <c r="P145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr"/>
       <c r="R145" t="inlineStr">
         <is>
           <t>Casa, 39.77 de área total, 38.60 de área privativa, 108.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11184,16 +11112,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1787700557135</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q146" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1787700557135.pdf</t>
-        </is>
-      </c>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr"/>
       <c r="R146" t="inlineStr">
         <is>
           <t>Apartamento, 45.88 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11260,16 +11180,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518325604</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q147" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518325604.pdf</t>
-        </is>
-      </c>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr"/>
       <c r="R147" t="inlineStr">
         <is>
           <t>Casa, 50.10 de área total, 50.10 de área privativa, 69.70 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -11337,11 +11249,7 @@
         </is>
       </c>
       <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701955078.pdf</t>
-        </is>
-      </c>
+      <c r="Q148" t="inlineStr"/>
       <c r="R148" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11408,16 +11316,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444414235560</t>
         </is>
       </c>
-      <c r="P149" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q149" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414235560.pdf</t>
-        </is>
-      </c>
+      <c r="P149" t="inlineStr"/>
+      <c r="Q149" t="inlineStr"/>
       <c r="R149" t="inlineStr">
         <is>
           <t>Apartamento, 63.98 de área total, 55.06 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11484,16 +11384,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518647563</t>
         </is>
       </c>
-      <c r="P150" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q150" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518647563.pdf</t>
-        </is>
-      </c>
+      <c r="P150" t="inlineStr"/>
+      <c r="Q150" t="inlineStr"/>
       <c r="R150" t="inlineStr">
         <is>
           <t>Apartamento, 44.95 de área total, 40.01 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -11560,16 +11452,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444423636724</t>
         </is>
       </c>
-      <c r="P151" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q151" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423636724.pdf</t>
-        </is>
-      </c>
+      <c r="P151" t="inlineStr"/>
+      <c r="Q151" t="inlineStr"/>
       <c r="R151" t="inlineStr">
         <is>
           <t>Apartamento, 49.30 de área total, 42.57 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11636,16 +11520,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444424287210</t>
         </is>
       </c>
-      <c r="P152" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q152" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444424287210.pdf</t>
-        </is>
-      </c>
+      <c r="P152" t="inlineStr"/>
+      <c r="Q152" t="inlineStr"/>
       <c r="R152" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 53.29 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11712,16 +11588,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555533967557</t>
         </is>
       </c>
-      <c r="P153" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q153" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555533967557.pdf</t>
-        </is>
-      </c>
+      <c r="P153" t="inlineStr"/>
+      <c r="Q153" t="inlineStr"/>
       <c r="R153" t="inlineStr">
         <is>
           <t>Apartamento, 62.64 de área total, 54.99 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11789,11 +11657,7 @@
         </is>
       </c>
       <c r="P154" t="inlineStr"/>
-      <c r="Q154" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010284141.pdf</t>
-        </is>
-      </c>
+      <c r="Q154" t="inlineStr"/>
       <c r="R154" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 547.75 de área privativa, 1468.00 de área do terreno,  5 qto(s), varanda, a.serv, WC, WC Emp, 2 sala(s), 1 lavabo(s), cozinha, Terraco.</t>
@@ -11860,16 +11724,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444407173466</t>
         </is>
       </c>
-      <c r="P155" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q155" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444407173466.pdf</t>
-        </is>
-      </c>
+      <c r="P155" t="inlineStr"/>
+      <c r="Q155" t="inlineStr"/>
       <c r="R155" t="inlineStr">
         <is>
           <t>Casa, 90.99 de área total, 90.99 de área privativa, 74.81 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), 1 lavabo(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11936,16 +11792,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1065020080212</t>
         </is>
       </c>
-      <c r="P156" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q156" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1065020080212.pdf</t>
-        </is>
-      </c>
+      <c r="P156" t="inlineStr"/>
+      <c r="Q156" t="inlineStr"/>
       <c r="R156" t="inlineStr">
         <is>
           <t>Apartamento, 98.25 de área total, 87.59 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, WC Emp, 1 sala(s), DCE, cozinha, 1 vaga(s) de garagem.</t>
@@ -12012,16 +11860,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444404619259</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q157" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404619259.pdf</t>
-        </is>
-      </c>
+      <c r="P157" t="inlineStr"/>
+      <c r="Q157" t="inlineStr"/>
       <c r="R157" t="inlineStr">
         <is>
           <t>Apartamento, 59.70 de área total, 59.70 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12089,11 +11929,7 @@
         </is>
       </c>
       <c r="P158" t="inlineStr"/>
-      <c r="Q158" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1555528553075.pdf</t>
-        </is>
-      </c>
+      <c r="Q158" t="inlineStr"/>
       <c r="R158" t="inlineStr">
         <is>
           <t>Casa, 410.32 de área total, 410.32 de área privativa, 528.00 de área do terreno,  3 qto(s), a.serv, WC, 4 sala(s), cozinha.</t>
@@ -12161,11 +11997,7 @@
         </is>
       </c>
       <c r="P159" t="inlineStr"/>
-      <c r="Q159" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418870180.pdf</t>
-        </is>
-      </c>
+      <c r="Q159" t="inlineStr"/>
       <c r="R159" t="inlineStr">
         <is>
           <t>Casa, 138.91 de área total, 51.72 de área privativa, 194.79 de área do terreno,  4 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12229,16 +12061,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=10286302</t>
         </is>
       </c>
-      <c r="P160" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q160" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010286302.pdf</t>
-        </is>
-      </c>
+      <c r="P160" t="inlineStr"/>
+      <c r="Q160" t="inlineStr"/>
       <c r="R160" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 70.07 de área privativa, 207.66 de área do terreno.</t>
@@ -12303,11 +12127,7 @@
         </is>
       </c>
       <c r="P161" t="inlineStr"/>
-      <c r="Q161" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418887481.pdf</t>
-        </is>
-      </c>
+      <c r="Q161" t="inlineStr"/>
       <c r="R161" t="inlineStr">
         <is>
           <t>Terreno, 0.00 de área total, 0.00 de área privativa, 480.00 de área do terreno.</t>
@@ -12374,16 +12194,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444423249372</t>
         </is>
       </c>
-      <c r="P162" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q162" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423249372.pdf</t>
-        </is>
-      </c>
+      <c r="P162" t="inlineStr"/>
+      <c r="Q162" t="inlineStr"/>
       <c r="R162" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 60.00 de área privativa, 120.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -12417,7 +12229,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 12:43</t>
+          <t>13/07/2026 às 13:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 16:19 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -9826,16 +9826,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787712957700</t>
         </is>
       </c>
-      <c r="P128" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q128" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787712957700.pdf</t>
-        </is>
-      </c>
+      <c r="P128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr"/>
       <c r="R128" t="inlineStr">
         <is>
           <t>Apartamento, 45.38 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), 1 sala(s), 1 vaga(s) de garagem.</t>
@@ -9902,16 +9894,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715863944</t>
         </is>
       </c>
-      <c r="P129" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q129" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715863944.pdf</t>
-        </is>
-      </c>
+      <c r="P129" t="inlineStr"/>
+      <c r="Q129" t="inlineStr"/>
       <c r="R129" t="inlineStr">
         <is>
           <t>Apartamento, 45.38 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9978,16 +9962,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444422964744</t>
         </is>
       </c>
-      <c r="P130" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q130" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444422964744.pdf</t>
-        </is>
-      </c>
+      <c r="P130" t="inlineStr"/>
+      <c r="Q130" t="inlineStr"/>
       <c r="R130" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 57.99 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10054,16 +10030,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703103958</t>
         </is>
       </c>
-      <c r="P131" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q131" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703103958.pdf</t>
-        </is>
-      </c>
+      <c r="P131" t="inlineStr"/>
+      <c r="Q131" t="inlineStr"/>
       <c r="R131" t="inlineStr">
         <is>
           <t>Apartamento, 51.50 de área total, 38.40 de área privativa, 0.00 de área do terreno,  1 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10130,16 +10098,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715235463</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q132" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715235463.pdf</t>
-        </is>
-      </c>
+      <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr"/>
       <c r="R132" t="inlineStr">
         <is>
           <t>Apartamento, 76.21 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10204,11 +10164,7 @@
         </is>
       </c>
       <c r="P133" t="inlineStr"/>
-      <c r="Q133" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444422825932.pdf</t>
-        </is>
-      </c>
+      <c r="Q133" t="inlineStr"/>
       <c r="R133" t="inlineStr">
         <is>
           <t>Terreno, 0.00 de área total, 0.00 de área privativa, 3328.92 de área do terreno.</t>
@@ -10275,16 +10231,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444422580050</t>
         </is>
       </c>
-      <c r="P134" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q134" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444422580050.pdf</t>
-        </is>
-      </c>
+      <c r="P134" t="inlineStr"/>
+      <c r="Q134" t="inlineStr"/>
       <c r="R134" t="inlineStr">
         <is>
           <t>Apartamento, 40.02 de área total, 36.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -10351,16 +10299,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715190850</t>
         </is>
       </c>
-      <c r="P135" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q135" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715190850.pdf</t>
-        </is>
-      </c>
+      <c r="P135" t="inlineStr"/>
+      <c r="Q135" t="inlineStr"/>
       <c r="R135" t="inlineStr">
         <is>
           <t>Apartamento, 52.70 de área total, 46.68 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10427,16 +10367,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716620441</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q136" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716620441.pdf</t>
-        </is>
-      </c>
+      <c r="P136" t="inlineStr"/>
+      <c r="Q136" t="inlineStr"/>
       <c r="R136" t="inlineStr">
         <is>
           <t>Apartamento, 72.39 de área total, 61.95 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12229,7 +12161,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 13:10</t>
+          <t>13/07/2026 às 13:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 16:47 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -9315,11 +9315,7 @@
         </is>
       </c>
       <c r="P121" t="inlineStr"/>
-      <c r="Q121" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703202964.pdf</t>
-        </is>
-      </c>
+      <c r="Q121" t="inlineStr"/>
       <c r="R121" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9387,11 +9383,7 @@
         </is>
       </c>
       <c r="P122" t="inlineStr"/>
-      <c r="Q122" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787709676569.pdf</t>
-        </is>
-      </c>
+      <c r="Q122" t="inlineStr"/>
       <c r="R122" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9458,16 +9450,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787700995319</t>
         </is>
       </c>
-      <c r="P123" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q123" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787700995319.pdf</t>
-        </is>
-      </c>
+      <c r="P123" t="inlineStr"/>
+      <c r="Q123" t="inlineStr"/>
       <c r="R123" t="inlineStr">
         <is>
           <t>Apartamento, 52.25 de área total, 43.54 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9535,11 +9519,7 @@
         </is>
       </c>
       <c r="P124" t="inlineStr"/>
-      <c r="Q124" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710407215.pdf</t>
-        </is>
-      </c>
+      <c r="Q124" t="inlineStr"/>
       <c r="R124" t="inlineStr">
         <is>
           <t>Apartamento, 58.42 de área total, 49.94 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9607,11 +9587,7 @@
         </is>
       </c>
       <c r="P125" t="inlineStr"/>
-      <c r="Q125" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404798498.pdf</t>
-        </is>
-      </c>
+      <c r="Q125" t="inlineStr"/>
       <c r="R125" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 51.43 de área privativa, 0.00 de área do terreno,  3 qto(s), 1 sala(s), cozinha.</t>
@@ -9679,11 +9655,7 @@
         </is>
       </c>
       <c r="P126" t="inlineStr"/>
-      <c r="Q126" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444406189855.pdf</t>
-        </is>
-      </c>
+      <c r="Q126" t="inlineStr"/>
       <c r="R126" t="inlineStr">
         <is>
           <t>Casa, 43.65 de área total, 43.65 de área privativa, 71.60 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -9750,16 +9722,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705100042</t>
         </is>
       </c>
-      <c r="P127" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q127" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705100042.pdf</t>
-        </is>
-      </c>
+      <c r="P127" t="inlineStr"/>
+      <c r="Q127" t="inlineStr"/>
       <c r="R127" t="inlineStr">
         <is>
           <t>Apartamento, 58.45 de área total, 52.86 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12161,7 +12125,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 13:35</t>
+          <t>13/07/2026 às 13:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 17:07 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -9315,7 +9315,11 @@
         </is>
       </c>
       <c r="P121" t="inlineStr"/>
-      <c r="Q121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703202964.pdf</t>
+        </is>
+      </c>
       <c r="R121" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9383,7 +9387,11 @@
         </is>
       </c>
       <c r="P122" t="inlineStr"/>
-      <c r="Q122" t="inlineStr"/>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787709676569.pdf</t>
+        </is>
+      </c>
       <c r="R122" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9450,8 +9458,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787700995319</t>
         </is>
       </c>
-      <c r="P123" t="inlineStr"/>
-      <c r="Q123" t="inlineStr"/>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787700995319.pdf</t>
+        </is>
+      </c>
       <c r="R123" t="inlineStr">
         <is>
           <t>Apartamento, 52.25 de área total, 43.54 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9519,7 +9535,11 @@
         </is>
       </c>
       <c r="P124" t="inlineStr"/>
-      <c r="Q124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710407215.pdf</t>
+        </is>
+      </c>
       <c r="R124" t="inlineStr">
         <is>
           <t>Apartamento, 58.42 de área total, 49.94 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9587,7 +9607,11 @@
         </is>
       </c>
       <c r="P125" t="inlineStr"/>
-      <c r="Q125" t="inlineStr"/>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404798498.pdf</t>
+        </is>
+      </c>
       <c r="R125" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 51.43 de área privativa, 0.00 de área do terreno,  3 qto(s), 1 sala(s), cozinha.</t>
@@ -9655,7 +9679,11 @@
         </is>
       </c>
       <c r="P126" t="inlineStr"/>
-      <c r="Q126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444406189855.pdf</t>
+        </is>
+      </c>
       <c r="R126" t="inlineStr">
         <is>
           <t>Casa, 43.65 de área total, 43.65 de área privativa, 71.60 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -9722,8 +9750,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705100042</t>
         </is>
       </c>
-      <c r="P127" t="inlineStr"/>
-      <c r="Q127" t="inlineStr"/>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705100042.pdf</t>
+        </is>
+      </c>
       <c r="R127" t="inlineStr">
         <is>
           <t>Apartamento, 58.45 de área total, 52.86 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9790,8 +9826,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787712957700</t>
         </is>
       </c>
-      <c r="P128" t="inlineStr"/>
-      <c r="Q128" t="inlineStr"/>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787712957700.pdf</t>
+        </is>
+      </c>
       <c r="R128" t="inlineStr">
         <is>
           <t>Apartamento, 45.38 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), 1 sala(s), 1 vaga(s) de garagem.</t>
@@ -9858,8 +9902,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715863944</t>
         </is>
       </c>
-      <c r="P129" t="inlineStr"/>
-      <c r="Q129" t="inlineStr"/>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715863944.pdf</t>
+        </is>
+      </c>
       <c r="R129" t="inlineStr">
         <is>
           <t>Apartamento, 45.38 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9926,8 +9978,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444422964744</t>
         </is>
       </c>
-      <c r="P130" t="inlineStr"/>
-      <c r="Q130" t="inlineStr"/>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444422964744.pdf</t>
+        </is>
+      </c>
       <c r="R130" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 57.99 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9994,8 +10054,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787703103958</t>
         </is>
       </c>
-      <c r="P131" t="inlineStr"/>
-      <c r="Q131" t="inlineStr"/>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703103958.pdf</t>
+        </is>
+      </c>
       <c r="R131" t="inlineStr">
         <is>
           <t>Apartamento, 51.50 de área total, 38.40 de área privativa, 0.00 de área do terreno,  1 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10062,8 +10130,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715235463</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr"/>
-      <c r="Q132" t="inlineStr"/>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715235463.pdf</t>
+        </is>
+      </c>
       <c r="R132" t="inlineStr">
         <is>
           <t>Apartamento, 76.21 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10128,7 +10204,11 @@
         </is>
       </c>
       <c r="P133" t="inlineStr"/>
-      <c r="Q133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444422825932.pdf</t>
+        </is>
+      </c>
       <c r="R133" t="inlineStr">
         <is>
           <t>Terreno, 0.00 de área total, 0.00 de área privativa, 3328.92 de área do terreno.</t>
@@ -10195,8 +10275,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444422580050</t>
         </is>
       </c>
-      <c r="P134" t="inlineStr"/>
-      <c r="Q134" t="inlineStr"/>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444422580050.pdf</t>
+        </is>
+      </c>
       <c r="R134" t="inlineStr">
         <is>
           <t>Apartamento, 40.02 de área total, 36.40 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -10263,8 +10351,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715190850</t>
         </is>
       </c>
-      <c r="P135" t="inlineStr"/>
-      <c r="Q135" t="inlineStr"/>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715190850.pdf</t>
+        </is>
+      </c>
       <c r="R135" t="inlineStr">
         <is>
           <t>Apartamento, 52.70 de área total, 46.68 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10331,8 +10427,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716620441</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr"/>
-      <c r="Q136" t="inlineStr"/>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716620441.pdf</t>
+        </is>
+      </c>
       <c r="R136" t="inlineStr">
         <is>
           <t>Apartamento, 72.39 de área total, 61.95 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10399,8 +10503,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715858002</t>
         </is>
       </c>
-      <c r="P137" t="inlineStr"/>
-      <c r="Q137" t="inlineStr"/>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715858002.pdf</t>
+        </is>
+      </c>
       <c r="R137" t="inlineStr">
         <is>
           <t>Apartamento, 49.15 de área total, 41.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10467,8 +10579,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444430740965</t>
         </is>
       </c>
-      <c r="P138" t="inlineStr"/>
-      <c r="Q138" t="inlineStr"/>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444430740965.pdf</t>
+        </is>
+      </c>
       <c r="R138" t="inlineStr">
         <is>
           <t>Apartamento, 59.43 de área total, 48.13 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10535,8 +10655,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787712390409</t>
         </is>
       </c>
-      <c r="P139" t="inlineStr"/>
-      <c r="Q139" t="inlineStr"/>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787712390409.pdf</t>
+        </is>
+      </c>
       <c r="R139" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10603,8 +10731,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714019724</t>
         </is>
       </c>
-      <c r="P140" t="inlineStr"/>
-      <c r="Q140" t="inlineStr"/>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00160326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714019724.pdf</t>
+        </is>
+      </c>
       <c r="R140" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10671,8 +10807,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714335693</t>
         </is>
       </c>
-      <c r="P141" t="inlineStr"/>
-      <c r="Q141" t="inlineStr"/>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714335693.pdf</t>
+        </is>
+      </c>
       <c r="R141" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10736,8 +10880,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716737225</t>
         </is>
       </c>
-      <c r="P142" t="inlineStr"/>
-      <c r="Q142" t="inlineStr"/>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716737225.pdf</t>
+        </is>
+      </c>
       <c r="R142" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 42.00 de área privativa, 78.00 de área do terreno.</t>
@@ -10804,8 +10956,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787718250838</t>
         </is>
       </c>
-      <c r="P143" t="inlineStr"/>
-      <c r="Q143" t="inlineStr"/>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00120326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787718250838.pdf</t>
+        </is>
+      </c>
       <c r="R143" t="inlineStr">
         <is>
           <t>Apartamento, 60.55 de área total, 55.26 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10872,8 +11032,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555532572478</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr"/>
-      <c r="Q144" t="inlineStr"/>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555532572478.pdf</t>
+        </is>
+      </c>
       <c r="R144" t="inlineStr">
         <is>
           <t>Apartamento, 60.24 de área total, 52.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10940,8 +11108,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444417159547</t>
         </is>
       </c>
-      <c r="P145" t="inlineStr"/>
-      <c r="Q145" t="inlineStr"/>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444417159547.pdf</t>
+        </is>
+      </c>
       <c r="R145" t="inlineStr">
         <is>
           <t>Casa, 39.77 de área total, 38.60 de área privativa, 108.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11008,8 +11184,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1787700557135</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr"/>
-      <c r="Q146" t="inlineStr"/>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1787700557135.pdf</t>
+        </is>
+      </c>
       <c r="R146" t="inlineStr">
         <is>
           <t>Apartamento, 45.88 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11076,8 +11260,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518325604</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr"/>
-      <c r="Q147" t="inlineStr"/>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518325604.pdf</t>
+        </is>
+      </c>
       <c r="R147" t="inlineStr">
         <is>
           <t>Casa, 50.10 de área total, 50.10 de área privativa, 69.70 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -12125,7 +12317,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 13:47</t>
+          <t>13/07/2026 às 14:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 18:03 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -11337,7 +11337,11 @@
         </is>
       </c>
       <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="inlineStr"/>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701955078.pdf</t>
+        </is>
+      </c>
       <c r="R148" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11404,8 +11408,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444414235560</t>
         </is>
       </c>
-      <c r="P149" t="inlineStr"/>
-      <c r="Q149" t="inlineStr"/>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414235560.pdf</t>
+        </is>
+      </c>
       <c r="R149" t="inlineStr">
         <is>
           <t>Apartamento, 63.98 de área total, 55.06 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11472,8 +11484,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518647563</t>
         </is>
       </c>
-      <c r="P150" t="inlineStr"/>
-      <c r="Q150" t="inlineStr"/>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518647563.pdf</t>
+        </is>
+      </c>
       <c r="R150" t="inlineStr">
         <is>
           <t>Apartamento, 44.95 de área total, 40.01 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -11540,8 +11560,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444423636724</t>
         </is>
       </c>
-      <c r="P151" t="inlineStr"/>
-      <c r="Q151" t="inlineStr"/>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423636724.pdf</t>
+        </is>
+      </c>
       <c r="R151" t="inlineStr">
         <is>
           <t>Apartamento, 49.30 de área total, 42.57 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11608,8 +11636,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444424287210</t>
         </is>
       </c>
-      <c r="P152" t="inlineStr"/>
-      <c r="Q152" t="inlineStr"/>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444424287210.pdf</t>
+        </is>
+      </c>
       <c r="R152" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 53.29 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11676,8 +11712,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555533967557</t>
         </is>
       </c>
-      <c r="P153" t="inlineStr"/>
-      <c r="Q153" t="inlineStr"/>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555533967557.pdf</t>
+        </is>
+      </c>
       <c r="R153" t="inlineStr">
         <is>
           <t>Apartamento, 62.64 de área total, 54.99 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11745,7 +11789,11 @@
         </is>
       </c>
       <c r="P154" t="inlineStr"/>
-      <c r="Q154" t="inlineStr"/>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010284141.pdf</t>
+        </is>
+      </c>
       <c r="R154" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 547.75 de área privativa, 1468.00 de área do terreno,  5 qto(s), varanda, a.serv, WC, WC Emp, 2 sala(s), 1 lavabo(s), cozinha, Terraco.</t>
@@ -11812,8 +11860,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444407173466</t>
         </is>
       </c>
-      <c r="P155" t="inlineStr"/>
-      <c r="Q155" t="inlineStr"/>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444407173466.pdf</t>
+        </is>
+      </c>
       <c r="R155" t="inlineStr">
         <is>
           <t>Casa, 90.99 de área total, 90.99 de área privativa, 74.81 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), 1 lavabo(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11880,8 +11936,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1065020080212</t>
         </is>
       </c>
-      <c r="P156" t="inlineStr"/>
-      <c r="Q156" t="inlineStr"/>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1065020080212.pdf</t>
+        </is>
+      </c>
       <c r="R156" t="inlineStr">
         <is>
           <t>Apartamento, 98.25 de área total, 87.59 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, WC Emp, 1 sala(s), DCE, cozinha, 1 vaga(s) de garagem.</t>
@@ -11948,8 +12012,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444404619259</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr"/>
-      <c r="Q157" t="inlineStr"/>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404619259.pdf</t>
+        </is>
+      </c>
       <c r="R157" t="inlineStr">
         <is>
           <t>Apartamento, 59.70 de área total, 59.70 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12017,7 +12089,11 @@
         </is>
       </c>
       <c r="P158" t="inlineStr"/>
-      <c r="Q158" t="inlineStr"/>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1555528553075.pdf</t>
+        </is>
+      </c>
       <c r="R158" t="inlineStr">
         <is>
           <t>Casa, 410.32 de área total, 410.32 de área privativa, 528.00 de área do terreno,  3 qto(s), a.serv, WC, 4 sala(s), cozinha.</t>
@@ -12085,7 +12161,11 @@
         </is>
       </c>
       <c r="P159" t="inlineStr"/>
-      <c r="Q159" t="inlineStr"/>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418870180.pdf</t>
+        </is>
+      </c>
       <c r="R159" t="inlineStr">
         <is>
           <t>Casa, 138.91 de área total, 51.72 de área privativa, 194.79 de área do terreno,  4 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12149,8 +12229,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=10286302</t>
         </is>
       </c>
-      <c r="P160" t="inlineStr"/>
-      <c r="Q160" t="inlineStr"/>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010286302.pdf</t>
+        </is>
+      </c>
       <c r="R160" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 70.07 de área privativa, 207.66 de área do terreno.</t>
@@ -12215,7 +12303,11 @@
         </is>
       </c>
       <c r="P161" t="inlineStr"/>
-      <c r="Q161" t="inlineStr"/>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418887481.pdf</t>
+        </is>
+      </c>
       <c r="R161" t="inlineStr">
         <is>
           <t>Terreno, 0.00 de área total, 0.00 de área privativa, 480.00 de área do terreno.</t>
@@ -12282,8 +12374,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444423249372</t>
         </is>
       </c>
-      <c r="P162" t="inlineStr"/>
-      <c r="Q162" t="inlineStr"/>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423249372.pdf</t>
+        </is>
+      </c>
       <c r="R162" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 60.00 de área privativa, 120.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -12317,7 +12417,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 14:07</t>
+          <t>13/07/2026 às 15:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 18:21 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -5083,11 +5083,7 @@
         </is>
       </c>
       <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710517002.pdf</t>
-        </is>
-      </c>
+      <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr">
         <is>
           <t>Apartamento, 45.87 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12417,7 +12413,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 15:13</t>
+          <t>13/07/2026 às 15:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 19:00 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -11932,16 +11932,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1065020080212</t>
         </is>
       </c>
-      <c r="P156" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q156" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1065020080212.pdf</t>
-        </is>
-      </c>
+      <c r="P156" t="inlineStr"/>
+      <c r="Q156" t="inlineStr"/>
       <c r="R156" t="inlineStr">
         <is>
           <t>Apartamento, 98.25 de área total, 87.59 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, WC Emp, 1 sala(s), DCE, cozinha, 1 vaga(s) de garagem.</t>
@@ -12008,16 +12000,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444404619259</t>
         </is>
       </c>
-      <c r="P157" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q157" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404619259.pdf</t>
-        </is>
-      </c>
+      <c r="P157" t="inlineStr"/>
+      <c r="Q157" t="inlineStr"/>
       <c r="R157" t="inlineStr">
         <is>
           <t>Apartamento, 59.70 de área total, 59.70 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12085,11 +12069,7 @@
         </is>
       </c>
       <c r="P158" t="inlineStr"/>
-      <c r="Q158" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1555528553075.pdf</t>
-        </is>
-      </c>
+      <c r="Q158" t="inlineStr"/>
       <c r="R158" t="inlineStr">
         <is>
           <t>Casa, 410.32 de área total, 410.32 de área privativa, 528.00 de área do terreno,  3 qto(s), a.serv, WC, 4 sala(s), cozinha.</t>
@@ -12157,11 +12137,7 @@
         </is>
       </c>
       <c r="P159" t="inlineStr"/>
-      <c r="Q159" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418870180.pdf</t>
-        </is>
-      </c>
+      <c r="Q159" t="inlineStr"/>
       <c r="R159" t="inlineStr">
         <is>
           <t>Casa, 138.91 de área total, 51.72 de área privativa, 194.79 de área do terreno,  4 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12225,16 +12201,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=10286302</t>
         </is>
       </c>
-      <c r="P160" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q160" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010286302.pdf</t>
-        </is>
-      </c>
+      <c r="P160" t="inlineStr"/>
+      <c r="Q160" t="inlineStr"/>
       <c r="R160" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 70.07 de área privativa, 207.66 de área do terreno.</t>
@@ -12299,11 +12267,7 @@
         </is>
       </c>
       <c r="P161" t="inlineStr"/>
-      <c r="Q161" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418887481.pdf</t>
-        </is>
-      </c>
+      <c r="Q161" t="inlineStr"/>
       <c r="R161" t="inlineStr">
         <is>
           <t>Terreno, 0.00 de área total, 0.00 de área privativa, 480.00 de área do terreno.</t>
@@ -12370,16 +12334,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444423249372</t>
         </is>
       </c>
-      <c r="P162" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q162" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423249372.pdf</t>
-        </is>
-      </c>
+      <c r="P162" t="inlineStr"/>
+      <c r="Q162" t="inlineStr"/>
       <c r="R162" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 60.00 de área privativa, 120.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -12413,7 +12369,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 15:31</t>
+          <t>13/07/2026 às 16:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 13/07/2026 19:08 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -11028,16 +11028,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555532572478</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q144" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555532572478.pdf</t>
-        </is>
-      </c>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
       <c r="R144" t="inlineStr">
         <is>
           <t>Apartamento, 60.24 de área total, 52.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11104,16 +11096,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444417159547</t>
         </is>
       </c>
-      <c r="P145" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q145" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444417159547.pdf</t>
-        </is>
-      </c>
+      <c r="P145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr"/>
       <c r="R145" t="inlineStr">
         <is>
           <t>Casa, 39.77 de área total, 38.60 de área privativa, 108.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11180,16 +11164,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1787700557135</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q146" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1787700557135.pdf</t>
-        </is>
-      </c>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr"/>
       <c r="R146" t="inlineStr">
         <is>
           <t>Apartamento, 45.88 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11256,16 +11232,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518325604</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q147" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518325604.pdf</t>
-        </is>
-      </c>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr"/>
       <c r="R147" t="inlineStr">
         <is>
           <t>Casa, 50.10 de área total, 50.10 de área privativa, 69.70 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -11333,11 +11301,7 @@
         </is>
       </c>
       <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701955078.pdf</t>
-        </is>
-      </c>
+      <c r="Q148" t="inlineStr"/>
       <c r="R148" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11404,16 +11368,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444414235560</t>
         </is>
       </c>
-      <c r="P149" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q149" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414235560.pdf</t>
-        </is>
-      </c>
+      <c r="P149" t="inlineStr"/>
+      <c r="Q149" t="inlineStr"/>
       <c r="R149" t="inlineStr">
         <is>
           <t>Apartamento, 63.98 de área total, 55.06 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11480,16 +11436,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518647563</t>
         </is>
       </c>
-      <c r="P150" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q150" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518647563.pdf</t>
-        </is>
-      </c>
+      <c r="P150" t="inlineStr"/>
+      <c r="Q150" t="inlineStr"/>
       <c r="R150" t="inlineStr">
         <is>
           <t>Apartamento, 44.95 de área total, 40.01 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -11556,16 +11504,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444423636724</t>
         </is>
       </c>
-      <c r="P151" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q151" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444423636724.pdf</t>
-        </is>
-      </c>
+      <c r="P151" t="inlineStr"/>
+      <c r="Q151" t="inlineStr"/>
       <c r="R151" t="inlineStr">
         <is>
           <t>Apartamento, 49.30 de área total, 42.57 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11632,16 +11572,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444424287210</t>
         </is>
       </c>
-      <c r="P152" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q152" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444424287210.pdf</t>
-        </is>
-      </c>
+      <c r="P152" t="inlineStr"/>
+      <c r="Q152" t="inlineStr"/>
       <c r="R152" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 53.29 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11708,16 +11640,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555533967557</t>
         </is>
       </c>
-      <c r="P153" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q153" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555533967557.pdf</t>
-        </is>
-      </c>
+      <c r="P153" t="inlineStr"/>
+      <c r="Q153" t="inlineStr"/>
       <c r="R153" t="inlineStr">
         <is>
           <t>Apartamento, 62.64 de área total, 54.99 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11785,11 +11709,7 @@
         </is>
       </c>
       <c r="P154" t="inlineStr"/>
-      <c r="Q154" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/0000010284141.pdf</t>
-        </is>
-      </c>
+      <c r="Q154" t="inlineStr"/>
       <c r="R154" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 547.75 de área privativa, 1468.00 de área do terreno,  5 qto(s), varanda, a.serv, WC, WC Emp, 2 sala(s), 1 lavabo(s), cozinha, Terraco.</t>
@@ -11856,16 +11776,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444407173466</t>
         </is>
       </c>
-      <c r="P155" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q155" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444407173466.pdf</t>
-        </is>
-      </c>
+      <c r="P155" t="inlineStr"/>
+      <c r="Q155" t="inlineStr"/>
       <c r="R155" t="inlineStr">
         <is>
           <t>Casa, 90.99 de área total, 90.99 de área privativa, 74.81 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), 1 lavabo(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -12369,7 +12281,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>13/07/2026 às 16:00</t>
+          <t>13/07/2026 às 16:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 19/07/2026 11:15 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -9693,7 +9693,11 @@
         </is>
       </c>
       <c r="P126" t="inlineStr"/>
-      <c r="Q126" t="inlineStr"/>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703188899.pdf</t>
+        </is>
+      </c>
       <c r="R126" t="inlineStr">
         <is>
           <t>Apartamento, 50.04 de área total, 43.61 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9761,7 +9765,11 @@
         </is>
       </c>
       <c r="P127" t="inlineStr"/>
-      <c r="Q127" t="inlineStr"/>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787703202964.pdf</t>
+        </is>
+      </c>
       <c r="R127" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9829,7 +9837,11 @@
         </is>
       </c>
       <c r="P128" t="inlineStr"/>
-      <c r="Q128" t="inlineStr"/>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787709676569.pdf</t>
+        </is>
+      </c>
       <c r="R128" t="inlineStr">
         <is>
           <t>Apartamento, 45.82 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9897,7 +9909,11 @@
         </is>
       </c>
       <c r="P129" t="inlineStr"/>
-      <c r="Q129" t="inlineStr"/>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787710407215.pdf</t>
+        </is>
+      </c>
       <c r="R129" t="inlineStr">
         <is>
           <t>Apartamento, 58.42 de área total, 49.94 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9965,7 +9981,11 @@
         </is>
       </c>
       <c r="P130" t="inlineStr"/>
-      <c r="Q130" t="inlineStr"/>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444404798498.pdf</t>
+        </is>
+      </c>
       <c r="R130" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 51.43 de área privativa, 0.00 de área do terreno,  3 qto(s), 1 sala(s), cozinha.</t>
@@ -12976,7 +12996,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>18/07/2026 às 08:11</t>
+          <t>19/07/2026 às 08:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 20/07/2026 12:23 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -3484,11 +3484,7 @@
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787706692334.pdf</t>
-        </is>
-      </c>
+      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>Apartamento, 46.27 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10053,7 +10049,11 @@
         </is>
       </c>
       <c r="P131" t="inlineStr"/>
-      <c r="Q131" t="inlineStr"/>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444406189855.pdf</t>
+        </is>
+      </c>
       <c r="R131" t="inlineStr">
         <is>
           <t>Casa, 43.65 de área total, 43.65 de área privativa, 71.60 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -10120,8 +10120,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787705100042</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr"/>
-      <c r="Q132" t="inlineStr"/>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705100042.pdf</t>
+        </is>
+      </c>
       <c r="R132" t="inlineStr">
         <is>
           <t>Apartamento, 58.45 de área total, 52.86 de área privativa, 0.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10188,8 +10196,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787712957700</t>
         </is>
       </c>
-      <c r="P133" t="inlineStr"/>
-      <c r="Q133" t="inlineStr"/>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00150326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787712957700.pdf</t>
+        </is>
+      </c>
       <c r="R133" t="inlineStr">
         <is>
           <t>Apartamento, 45.38 de área total, 38.40 de área privativa, 0.00 de área do terreno,  2 qto(s), 1 sala(s), 1 vaga(s) de garagem.</t>
@@ -12996,7 +13012,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>19/07/2026 às 08:15</t>
+          <t>20/07/2026 às 09:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 21/07/2026 15:26 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -755,11 +755,7 @@
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705420250.pdf</t>
-        </is>
-      </c>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>Apartamento, 101.65 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -1420,11 +1416,7 @@
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702551558.pdf</t>
-        </is>
-      </c>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -9913,8 +9905,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444419971338</t>
         </is>
       </c>
-      <c r="P129" t="inlineStr"/>
-      <c r="Q129" t="inlineStr"/>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444419971338.pdf</t>
+        </is>
+      </c>
       <c r="R129" t="inlineStr">
         <is>
           <t>Casa, 60.00 de área total, 60.00 de área privativa, 192.00 de área do terreno,  3 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -9981,8 +9981,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715190850</t>
         </is>
       </c>
-      <c r="P130" t="inlineStr"/>
-      <c r="Q130" t="inlineStr"/>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715190850.pdf</t>
+        </is>
+      </c>
       <c r="R130" t="inlineStr">
         <is>
           <t>Apartamento, 52.70 de área total, 46.68 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10049,8 +10057,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716620441</t>
         </is>
       </c>
-      <c r="P131" t="inlineStr"/>
-      <c r="Q131" t="inlineStr"/>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716620441.pdf</t>
+        </is>
+      </c>
       <c r="R131" t="inlineStr">
         <is>
           <t>Apartamento, 72.39 de área total, 61.95 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10117,8 +10133,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715985985</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr"/>
-      <c r="Q132" t="inlineStr"/>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00240326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715985985.pdf</t>
+        </is>
+      </c>
       <c r="R132" t="inlineStr">
         <is>
           <t>Apartamento, 46.02 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10185,8 +10209,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716013782</t>
         </is>
       </c>
-      <c r="P133" t="inlineStr"/>
-      <c r="Q133" t="inlineStr"/>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00240326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716013782.pdf</t>
+        </is>
+      </c>
       <c r="R133" t="inlineStr">
         <is>
           <t>Apartamento, 46.02 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10253,8 +10285,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716933091</t>
         </is>
       </c>
-      <c r="P134" t="inlineStr"/>
-      <c r="Q134" t="inlineStr"/>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716933091.pdf</t>
+        </is>
+      </c>
       <c r="R134" t="inlineStr">
         <is>
           <t>Apartamento, 45.67 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10321,8 +10361,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715858002</t>
         </is>
       </c>
-      <c r="P135" t="inlineStr"/>
-      <c r="Q135" t="inlineStr"/>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715858002.pdf</t>
+        </is>
+      </c>
       <c r="R135" t="inlineStr">
         <is>
           <t>Apartamento, 49.15 de área total, 41.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10389,8 +10437,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444430740965</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr"/>
-      <c r="Q136" t="inlineStr"/>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444430740965.pdf</t>
+        </is>
+      </c>
       <c r="R136" t="inlineStr">
         <is>
           <t>Apartamento, 59.43 de área total, 48.13 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10457,8 +10513,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714335693</t>
         </is>
       </c>
-      <c r="P137" t="inlineStr"/>
-      <c r="Q137" t="inlineStr"/>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714335693.pdf</t>
+        </is>
+      </c>
       <c r="R137" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10525,8 +10589,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714993259</t>
         </is>
       </c>
-      <c r="P138" t="inlineStr"/>
-      <c r="Q138" t="inlineStr"/>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714993259.pdf</t>
+        </is>
+      </c>
       <c r="R138" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10590,8 +10662,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716737225</t>
         </is>
       </c>
-      <c r="P139" t="inlineStr"/>
-      <c r="Q139" t="inlineStr"/>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716737225.pdf</t>
+        </is>
+      </c>
       <c r="R139" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 42.00 de área privativa, 78.00 de área do terreno.</t>
@@ -10658,8 +10738,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444414053667</t>
         </is>
       </c>
-      <c r="P140" t="inlineStr"/>
-      <c r="Q140" t="inlineStr"/>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00240326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414053667.pdf</t>
+        </is>
+      </c>
       <c r="R140" t="inlineStr">
         <is>
           <t>Casa, 51.00 de área total, 51.00 de área privativa, 576.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10723,8 +10811,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444417549572</t>
         </is>
       </c>
-      <c r="P141" t="inlineStr"/>
-      <c r="Q141" t="inlineStr"/>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444417549572.pdf</t>
+        </is>
+      </c>
       <c r="R141" t="inlineStr">
         <is>
           <t>Casa, 36.49 de área total, 36.49 de área privativa, 67.50 de área do terreno.</t>
@@ -10791,8 +10887,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444417159547</t>
         </is>
       </c>
-      <c r="P142" t="inlineStr"/>
-      <c r="Q142" t="inlineStr"/>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444417159547.pdf</t>
+        </is>
+      </c>
       <c r="R142" t="inlineStr">
         <is>
           <t>Casa, 39.77 de área total, 38.60 de área privativa, 108.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10859,8 +10963,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1787700557135</t>
         </is>
       </c>
-      <c r="P143" t="inlineStr"/>
-      <c r="Q143" t="inlineStr"/>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1787700557135.pdf</t>
+        </is>
+      </c>
       <c r="R143" t="inlineStr">
         <is>
           <t>Apartamento, 45.88 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10927,8 +11039,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518325604</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr"/>
-      <c r="Q144" t="inlineStr"/>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518325604.pdf</t>
+        </is>
+      </c>
       <c r="R144" t="inlineStr">
         <is>
           <t>Casa, 50.10 de área total, 50.10 de área privativa, 69.70 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10996,7 +11116,11 @@
         </is>
       </c>
       <c r="P145" t="inlineStr"/>
-      <c r="Q145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701955078.pdf</t>
+        </is>
+      </c>
       <c r="R145" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11063,8 +11187,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444414235560</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr"/>
-      <c r="Q146" t="inlineStr"/>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414235560.pdf</t>
+        </is>
+      </c>
       <c r="R146" t="inlineStr">
         <is>
           <t>Apartamento, 63.98 de área total, 55.06 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11131,8 +11263,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518647563</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr"/>
-      <c r="Q147" t="inlineStr"/>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518647563.pdf</t>
+        </is>
+      </c>
       <c r="R147" t="inlineStr">
         <is>
           <t>Apartamento, 44.95 de área total, 40.01 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -11199,8 +11339,16 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444418577210</t>
         </is>
       </c>
-      <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="inlineStr"/>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418577210.pdf</t>
+        </is>
+      </c>
       <c r="R148" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 73.20 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -11843,7 +11991,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>21/07/2026 às 08:53</t>
+          <t>21/07/2026 às 12:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 21/07/2026 17:32 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -755,7 +755,11 @@
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787705420250.pdf</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>Apartamento, 101.65 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -1416,7 +1420,11 @@
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787702551558.pdf</t>
+        </is>
+      </c>
       <c r="R13" t="inlineStr">
         <is>
           <t>Apartamento, 45.91 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10887,16 +10895,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444417159547</t>
         </is>
       </c>
-      <c r="P142" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q142" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444417159547.pdf</t>
-        </is>
-      </c>
+      <c r="P142" t="inlineStr"/>
+      <c r="Q142" t="inlineStr"/>
       <c r="R142" t="inlineStr">
         <is>
           <t>Casa, 39.77 de área total, 38.60 de área privativa, 108.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10963,16 +10963,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1787700557135</t>
         </is>
       </c>
-      <c r="P143" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q143" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1787700557135.pdf</t>
-        </is>
-      </c>
+      <c r="P143" t="inlineStr"/>
+      <c r="Q143" t="inlineStr"/>
       <c r="R143" t="inlineStr">
         <is>
           <t>Apartamento, 45.88 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11039,16 +11031,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518325604</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q144" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518325604.pdf</t>
-        </is>
-      </c>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
       <c r="R144" t="inlineStr">
         <is>
           <t>Casa, 50.10 de área total, 50.10 de área privativa, 69.70 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -11116,11 +11100,7 @@
         </is>
       </c>
       <c r="P145" t="inlineStr"/>
-      <c r="Q145" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787701955078.pdf</t>
-        </is>
-      </c>
+      <c r="Q145" t="inlineStr"/>
       <c r="R145" t="inlineStr">
         <is>
           <t>Apartamento, 0.00 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11187,16 +11167,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444414235560</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q146" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414235560.pdf</t>
-        </is>
-      </c>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr"/>
       <c r="R146" t="inlineStr">
         <is>
           <t>Apartamento, 63.98 de área total, 55.06 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -11263,16 +11235,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8555518647563</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00190326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q147" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8555518647563.pdf</t>
-        </is>
-      </c>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr"/>
       <c r="R147" t="inlineStr">
         <is>
           <t>Apartamento, 44.95 de área total, 40.01 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha.</t>
@@ -11339,16 +11303,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444418577210</t>
         </is>
       </c>
-      <c r="P148" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q148" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444418577210.pdf</t>
-        </is>
-      </c>
+      <c r="P148" t="inlineStr"/>
+      <c r="Q148" t="inlineStr"/>
       <c r="R148" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 73.20 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -11991,7 +11947,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>21/07/2026 às 12:26</t>
+          <t>21/07/2026 às 14:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza vitrine — 21/07/2026 20:37 UTC
</commit_message>
<xml_diff>
--- a/docs/imoveis.xlsx
+++ b/docs/imoveis.xlsx
@@ -10065,16 +10065,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716620441</t>
         </is>
       </c>
-      <c r="P131" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q131" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716620441.pdf</t>
-        </is>
-      </c>
+      <c r="P131" t="inlineStr"/>
+      <c r="Q131" t="inlineStr"/>
       <c r="R131" t="inlineStr">
         <is>
           <t>Apartamento, 72.39 de área total, 61.95 de área privativa, 0.00 de área do terreno,  2 qto(s), varanda, a.serv, WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10141,16 +10133,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715985985</t>
         </is>
       </c>
-      <c r="P132" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00240326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q132" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715985985.pdf</t>
-        </is>
-      </c>
+      <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr"/>
       <c r="R132" t="inlineStr">
         <is>
           <t>Apartamento, 46.02 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10217,16 +10201,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716013782</t>
         </is>
       </c>
-      <c r="P133" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00240326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q133" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716013782.pdf</t>
-        </is>
-      </c>
+      <c r="P133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr"/>
       <c r="R133" t="inlineStr">
         <is>
           <t>Apartamento, 46.02 de área total, 40.31 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10293,16 +10269,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716933091</t>
         </is>
       </c>
-      <c r="P134" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q134" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716933091.pdf</t>
-        </is>
-      </c>
+      <c r="P134" t="inlineStr"/>
+      <c r="Q134" t="inlineStr"/>
       <c r="R134" t="inlineStr">
         <is>
           <t>Apartamento, 45.67 de área total, 40.00 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10369,16 +10337,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787715858002</t>
         </is>
       </c>
-      <c r="P135" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00200326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q135" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787715858002.pdf</t>
-        </is>
-      </c>
+      <c r="P135" t="inlineStr"/>
+      <c r="Q135" t="inlineStr"/>
       <c r="R135" t="inlineStr">
         <is>
           <t>Apartamento, 49.15 de área total, 41.60 de área privativa, 0.00 de área do terreno,  2 qto(s), WC, 1 sala(s), cozinha, 1 vaga(s) de garagem.</t>
@@ -10445,16 +10405,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444430740965</t>
         </is>
       </c>
-      <c r="P136" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00180326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q136" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444430740965.pdf</t>
-        </is>
-      </c>
+      <c r="P136" t="inlineStr"/>
+      <c r="Q136" t="inlineStr"/>
       <c r="R136" t="inlineStr">
         <is>
           <t>Apartamento, 59.43 de área total, 48.13 de área privativa, 0.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10521,16 +10473,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714335693</t>
         </is>
       </c>
-      <c r="P137" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00170326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q137" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714335693.pdf</t>
-        </is>
-      </c>
+      <c r="P137" t="inlineStr"/>
+      <c r="Q137" t="inlineStr"/>
       <c r="R137" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10597,16 +10541,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787714993259</t>
         </is>
       </c>
-      <c r="P138" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q138" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787714993259.pdf</t>
-        </is>
-      </c>
+      <c r="P138" t="inlineStr"/>
+      <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr">
         <is>
           <t>Casa, 42.00 de área total, 42.00 de área privativa, 78.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10670,16 +10606,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8787716737225</t>
         </is>
       </c>
-      <c r="P139" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00140326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q139" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8787716737225.pdf</t>
-        </is>
-      </c>
+      <c r="P139" t="inlineStr"/>
+      <c r="Q139" t="inlineStr"/>
       <c r="R139" t="inlineStr">
         <is>
           <t>Casa, 0.00 de área total, 42.00 de área privativa, 78.00 de área do terreno.</t>
@@ -10746,16 +10674,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=1444414053667</t>
         </is>
       </c>
-      <c r="P140" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00240326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q140" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/1444414053667.pdf</t>
-        </is>
-      </c>
+      <c r="P140" t="inlineStr"/>
+      <c r="Q140" t="inlineStr"/>
       <c r="R140" t="inlineStr">
         <is>
           <t>Casa, 51.00 de área total, 51.00 de área privativa, 576.00 de área do terreno,  2 qto(s), a.serv, WC, 1 sala(s), cozinha.</t>
@@ -10819,16 +10739,8 @@
           <t>https://venda-imoveis.caixa.gov.br/sistema/detalhe-imovel.asp?hdnimovel=8444417549572</t>
         </is>
       </c>
-      <c r="P141" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/EA00220326CPVERE.PDF</t>
-        </is>
-      </c>
-      <c r="Q141" t="inlineStr">
-        <is>
-          <t>https://venda-imoveis.caixa.gov.br/editais/matricula/PR/8444417549572.pdf</t>
-        </is>
-      </c>
+      <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr"/>
       <c r="R141" t="inlineStr">
         <is>
           <t>Casa, 36.49 de área total, 36.49 de área privativa, 67.50 de área do terreno.</t>
@@ -11947,7 +11859,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>21/07/2026 às 14:32</t>
+          <t>21/07/2026 às 17:37</t>
         </is>
       </c>
     </row>

</xml_diff>